<commit_message>
Complete Hungarian Method MATLAB case study with code breakdown and 100x100 clock-time benchmarks
</commit_message>
<xml_diff>
--- a/Electic Scooter Fleet/INDE 460 - Cost Final Project.xlsx
+++ b/Electic Scooter Fleet/INDE 460 - Cost Final Project.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/evdawgsmac/LocalFiles/P_Path/Job Search/Project Portfolio/Electic Scooter Fleet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{252678D2-BE56-D54C-9B1F-C0DE33D90C88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2C356E1-FBD8-8F40-A7B3-15F8E1037979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17500" activeTab="7" xr2:uid="{4E1F7FCE-C5AE-4A76-87F8-0DC26954148D}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17500" activeTab="8" xr2:uid="{4E1F7FCE-C5AE-4A76-87F8-0DC26954148D}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Details" sheetId="1" r:id="rId1"/>
@@ -1297,7 +1297,7 @@
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="176">
+  <cellXfs count="173">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1591,152 +1591,147 @@
     </xf>
     <xf numFmtId="165" fontId="12" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="44" fontId="8" fillId="0" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="8" fillId="0" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="11" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="8" fillId="0" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="8" fillId="0" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1784,11 +1779,9 @@
           <a:lstStyle/>
           <a:p>
             <a:pPr>
-              <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" cap="none" baseline="0">
+              <a:defRPr sz="2000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="lt1">
-                    <a:lumMod val="85000"/>
-                  </a:schemeClr>
+                  <a:schemeClr val="tx2"/>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
                 <a:ea typeface="+mn-ea"/>
@@ -1796,864 +1789,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US"/>
-              <a:t>Discounted Project Value over time ($180 Annual Fee &amp; 12% Avg Adoption)</a:t>
-            </a:r>
-          </a:p>
-          <a:p>
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:rich>
-      </c:tx>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="1" i="0" u="none" strike="noStrike" kern="1200" cap="none" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="lt1">
-                  <a:lumMod val="85000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="en-US"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
-    <c:autoTitleDeleted val="0"/>
-    <c:plotArea>
-      <c:layout>
-        <c:manualLayout>
-          <c:layoutTarget val="inner"/>
-          <c:xMode val="edge"/>
-          <c:yMode val="edge"/>
-          <c:x val="0.11411803281482112"/>
-          <c:y val="4.9125325883209045E-2"/>
-          <c:w val="0.86145058818682385"/>
-          <c:h val="0.87881930559528698"/>
-        </c:manualLayout>
-      </c:layout>
-      <c:lineChart>
-        <c:grouping val="standard"/>
-        <c:varyColors val="0"/>
-        <c:ser>
-          <c:idx val="0"/>
-          <c:order val="0"/>
-          <c:tx>
-            <c:strRef>
-              <c:f>Cashflow!$L$1</c:f>
-              <c:strCache>
-                <c:ptCount val="1"/>
-                <c:pt idx="0">
-                  <c:v>Discounted Project Value</c:v>
-                </c:pt>
-              </c:strCache>
-            </c:strRef>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="28575" cap="rnd">
-              <a:solidFill>
-                <a:srgbClr val="FFFF00"/>
-              </a:solidFill>
-            </a:ln>
-            <a:effectLst>
-              <a:glow rad="139700">
-                <a:schemeClr val="accent1">
-                  <a:satMod val="175000"/>
-                  <a:alpha val="14000"/>
-                </a:schemeClr>
-              </a:glow>
-            </a:effectLst>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="none"/>
-          </c:marker>
-          <c:cat>
-            <c:numRef>
-              <c:f>Cashflow!$B$2:$B$62</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="61"/>
-                <c:pt idx="0">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>1</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>2</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>3</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>4</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>5</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>6</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>7</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>8</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>9</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>10</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>11</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>12</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>13</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>14</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>15</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>16</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>17</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>18</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>19</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>20</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>21</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>22</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>23</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>24</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>25</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>26</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>27</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>28</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>29</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>30</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>31</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>32</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>33</c:v>
-                </c:pt>
-                <c:pt idx="34">
-                  <c:v>34</c:v>
-                </c:pt>
-                <c:pt idx="35">
-                  <c:v>35</c:v>
-                </c:pt>
-                <c:pt idx="36">
-                  <c:v>36</c:v>
-                </c:pt>
-                <c:pt idx="37">
-                  <c:v>37</c:v>
-                </c:pt>
-                <c:pt idx="38">
-                  <c:v>38</c:v>
-                </c:pt>
-                <c:pt idx="39">
-                  <c:v>39</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>40</c:v>
-                </c:pt>
-                <c:pt idx="41">
-                  <c:v>41</c:v>
-                </c:pt>
-                <c:pt idx="42">
-                  <c:v>42</c:v>
-                </c:pt>
-                <c:pt idx="43">
-                  <c:v>43</c:v>
-                </c:pt>
-                <c:pt idx="44">
-                  <c:v>44</c:v>
-                </c:pt>
-                <c:pt idx="45">
-                  <c:v>45</c:v>
-                </c:pt>
-                <c:pt idx="46">
-                  <c:v>46</c:v>
-                </c:pt>
-                <c:pt idx="47">
-                  <c:v>47</c:v>
-                </c:pt>
-                <c:pt idx="48">
-                  <c:v>48</c:v>
-                </c:pt>
-                <c:pt idx="49">
-                  <c:v>49</c:v>
-                </c:pt>
-                <c:pt idx="50">
-                  <c:v>50</c:v>
-                </c:pt>
-                <c:pt idx="51">
-                  <c:v>51</c:v>
-                </c:pt>
-                <c:pt idx="52">
-                  <c:v>52</c:v>
-                </c:pt>
-                <c:pt idx="53">
-                  <c:v>53</c:v>
-                </c:pt>
-                <c:pt idx="54">
-                  <c:v>54</c:v>
-                </c:pt>
-                <c:pt idx="55">
-                  <c:v>55</c:v>
-                </c:pt>
-                <c:pt idx="56">
-                  <c:v>56</c:v>
-                </c:pt>
-                <c:pt idx="57">
-                  <c:v>57</c:v>
-                </c:pt>
-                <c:pt idx="58">
-                  <c:v>58</c:v>
-                </c:pt>
-                <c:pt idx="59">
-                  <c:v>59</c:v>
-                </c:pt>
-                <c:pt idx="60">
-                  <c:v>60</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:cat>
-          <c:val>
-            <c:numRef>
-              <c:f>Cashflow!$L$2:$L$62</c:f>
-              <c:numCache>
-                <c:formatCode>"$"#,##0.00</c:formatCode>
-                <c:ptCount val="61"/>
-                <c:pt idx="0">
-                  <c:v>77361.53</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>61425.636857690537</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>45565.086703934605</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>29779.49181681835</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>14068.466620520434</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>-1568.3723272302159</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>-17131.406347620781</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>-32621.014653145292</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>-48037.574359920254</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>-63381.460499925859</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>-78653.046033172839</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>-93852.701859795663</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>97381.452026374813</c:v>
-                </c:pt>
-                <c:pt idx="13">
-                  <c:v>82324.551092074093</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>67338.479403414312</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>52422.874180291015</c:v>
-                </c:pt>
-                <c:pt idx="16">
-                  <c:v>37577.37464309913</c:v>
-                </c:pt>
-                <c:pt idx="17">
-                  <c:v>22801.622001072326</c:v>
-                </c:pt>
-                <c:pt idx="18">
-                  <c:v>8095.2594406929275</c:v>
-                </c:pt>
-                <c:pt idx="19">
-                  <c:v>-6542.0678858279716</c:v>
-                </c:pt>
-                <c:pt idx="20">
-                  <c:v>-21110.712872000906</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>-35611.026468438926</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>-50043.357694169885</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>-64408.053647880268</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>119058.36230358796</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>104827.90322341322</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>90664.049529826894</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>76566.461694423051</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>62534.802053929248</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>48568.734799364283</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>34667.925965261427</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>20832.043418956731</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>7060.7568499420158</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>-6646.2622407178569</c:v>
-                </c:pt>
-                <c:pt idx="34">
-                  <c:v>-20289.340550903842</c:v>
-                </c:pt>
-                <c:pt idx="35">
-                  <c:v>-33868.80298789806</c:v>
-                </c:pt>
-                <c:pt idx="36">
-                  <c:v>142138.68990129122</c:v>
-                </c:pt>
-                <c:pt idx="37">
-                  <c:v>133951.91969095633</c:v>
-                </c:pt>
-                <c:pt idx="38">
-                  <c:v>125794.13353427428</c:v>
-                </c:pt>
-                <c:pt idx="39">
-                  <c:v>117665.22881747375</c:v>
-                </c:pt>
-                <c:pt idx="40">
-                  <c:v>109565.10329007238</c:v>
-                </c:pt>
-                <c:pt idx="41">
-                  <c:v>101493.65506359056</c:v>
-                </c:pt>
-                <c:pt idx="42">
-                  <c:v>93450.782610269802</c:v>
-                </c:pt>
-                <c:pt idx="43">
-                  <c:v>85436.384761795736</c:v>
-                </c:pt>
-                <c:pt idx="44">
-                  <c:v>77450.360708025502</c:v>
-                </c:pt>
-                <c:pt idx="45">
-                  <c:v>69492.609995719657</c:v>
-                </c:pt>
-                <c:pt idx="46">
-                  <c:v>61563.032527278665</c:v>
-                </c:pt>
-                <c:pt idx="47">
-                  <c:v>53661.528559483821</c:v>
-                </c:pt>
-                <c:pt idx="48">
-                  <c:v>227414.84200814046</c:v>
-                </c:pt>
-                <c:pt idx="49">
-                  <c:v>219569.18722323619</c:v>
-                </c:pt>
-                <c:pt idx="50">
-                  <c:v>211751.30882308257</c:v>
-                </c:pt>
-                <c:pt idx="51">
-                  <c:v>203961.10846948205</c:v>
-                </c:pt>
-                <c:pt idx="52">
-                  <c:v>196198.48817238907</c:v>
-                </c:pt>
-                <c:pt idx="53">
-                  <c:v>188463.35028867732</c:v>
-                </c:pt>
-                <c:pt idx="54">
-                  <c:v>180755.5975209116</c:v>
-                </c:pt>
-                <c:pt idx="55">
-                  <c:v>173075.13291612396</c:v>
-                </c:pt>
-                <c:pt idx="56">
-                  <c:v>165421.85986459412</c:v>
-                </c:pt>
-                <c:pt idx="57">
-                  <c:v>157795.68209863434</c:v>
-                </c:pt>
-                <c:pt idx="58">
-                  <c:v>150196.5036913784</c:v>
-                </c:pt>
-                <c:pt idx="59">
-                  <c:v>142624.22905557498</c:v>
-                </c:pt>
-                <c:pt idx="60">
-                  <c:v>185448.79524921341</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:val>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-321E-A946-936B-6438C5B41BEC}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:dLbls>
-          <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
-          <c:showCatName val="0"/>
-          <c:showSerName val="0"/>
-          <c:showPercent val="0"/>
-          <c:showBubbleSize val="0"/>
-        </c:dLbls>
-        <c:smooth val="0"/>
-        <c:axId val="597914751"/>
-        <c:axId val="597908479"/>
-      </c:lineChart>
-      <c:catAx>
-        <c:axId val="597914751"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="b"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:gradFill>
-                <a:gsLst>
-                  <a:gs pos="100000">
-                    <a:schemeClr val="dk1">
-                      <a:lumMod val="75000"/>
-                      <a:lumOff val="25000"/>
-                    </a:schemeClr>
-                  </a:gs>
-                  <a:gs pos="0">
-                    <a:schemeClr val="dk1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:gs>
-                </a:gsLst>
-                <a:lin ang="5400000" scaled="0"/>
-              </a:gradFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="lt1">
-                        <a:lumMod val="75000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr lang="en-US" sz="1600"/>
-                  <a:t>Month</a:t>
-                </a:r>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:layout>
-            <c:manualLayout>
-              <c:xMode val="edge"/>
-              <c:yMode val="edge"/>
-              <c:x val="0.50361256708343938"/>
-              <c:y val="0.96558484305651748"/>
-            </c:manualLayout>
-          </c:layout>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="900" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="lt1">
-                      <a:lumMod val="75000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
-        </c:title>
-        <c:numFmt formatCode="General" sourceLinked="0"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="low"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:solidFill>
-              <a:schemeClr val="bg1"/>
-            </a:solidFill>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="bg1"/>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="597908479"/>
-        <c:crosses val="autoZero"/>
-        <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
-        <c:lblOffset val="100"/>
-        <c:tickMarkSkip val="1"/>
-        <c:noMultiLvlLbl val="0"/>
-      </c:catAx>
-      <c:valAx>
-        <c:axId val="597908479"/>
-        <c:scaling>
-          <c:orientation val="minMax"/>
-        </c:scaling>
-        <c:delete val="0"/>
-        <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:gradFill>
-                <a:gsLst>
-                  <a:gs pos="100000">
-                    <a:schemeClr val="dk1">
-                      <a:lumMod val="75000"/>
-                      <a:lumOff val="25000"/>
-                    </a:schemeClr>
-                  </a:gs>
-                  <a:gs pos="0">
-                    <a:schemeClr val="dk1">
-                      <a:lumMod val="65000"/>
-                      <a:lumOff val="35000"/>
-                    </a:schemeClr>
-                  </a:gs>
-                </a:gsLst>
-                <a:lin ang="5400000" scaled="0"/>
-              </a:gradFill>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
-        <c:title>
-          <c:tx>
-            <c:rich>
-              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-              <a:lstStyle/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                    <a:solidFill>
-                      <a:schemeClr val="lt1">
-                        <a:lumMod val="75000"/>
-                      </a:schemeClr>
-                    </a:solidFill>
-                    <a:latin typeface="+mn-lt"/>
-                    <a:ea typeface="+mn-ea"/>
-                    <a:cs typeface="+mn-cs"/>
-                  </a:defRPr>
-                </a:pPr>
-                <a:r>
-                  <a:rPr lang="en-US" sz="1600"/>
-                  <a:t>Project Value</a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="en-US" sz="1600" baseline="0"/>
-                  <a:t> ($)</a:t>
-                </a:r>
-                <a:endParaRPr lang="en-US" sz="1600"/>
-              </a:p>
-            </c:rich>
-          </c:tx>
-          <c:layout>
-            <c:manualLayout>
-              <c:xMode val="edge"/>
-              <c:yMode val="edge"/>
-              <c:x val="3.8430875424135681E-2"/>
-              <c:y val="0.42395693795968348"/>
-            </c:manualLayout>
-          </c:layout>
-          <c:overlay val="0"/>
-          <c:spPr>
-            <a:noFill/>
-            <a:ln>
-              <a:noFill/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:txPr>
-            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:pPr>
-                <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                  <a:solidFill>
-                    <a:schemeClr val="lt1">
-                      <a:lumMod val="75000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:pPr>
-              <a:endParaRPr lang="en-US"/>
-            </a:p>
-          </c:txPr>
-        </c:title>
-        <c:numFmt formatCode="&quot;$&quot;#,##0.00" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
-        <c:minorTickMark val="none"/>
-        <c:tickLblPos val="low"/>
-        <c:spPr>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:effectLst/>
-        </c:spPr>
-        <c:txPr>
-          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="lt1">
-                    <a:lumMod val="75000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:endParaRPr lang="en-US"/>
-          </a:p>
-        </c:txPr>
-        <c:crossAx val="597914751"/>
-        <c:crossesAt val="6"/>
-        <c:crossBetween val="between"/>
-      </c:valAx>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-    </c:plotArea>
-    <c:plotVisOnly val="1"/>
-    <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
-  </c:chart>
-  <c:spPr>
-    <a:solidFill>
-      <a:schemeClr val="dk1">
-        <a:lumMod val="75000"/>
-        <a:lumOff val="25000"/>
-      </a:schemeClr>
-    </a:solidFill>
-    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:round/>
-    </a:ln>
-    <a:effectLst/>
-  </c:spPr>
-  <c:txPr>
-    <a:bodyPr/>
-    <a:lstStyle/>
-    <a:p>
-      <a:pPr>
-        <a:defRPr/>
-      </a:pPr>
-      <a:endParaRPr lang="en-US"/>
-    </a:p>
-  </c:txPr>
-  <c:printSettings>
-    <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
-  </c:printSettings>
-</c:chartSpace>
-</file>
-
-<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
-  <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
-  <c:roundedCorners val="0"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
-    </mc:Choice>
-    <mc:Fallback>
-      <c:style val="2"/>
-    </mc:Fallback>
-  </mc:AlternateContent>
-  <c:chart>
-    <c:title>
-      <c:tx>
-        <c:rich>
-          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr>
-              <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="100" baseline="0">
-                <a:solidFill>
-                  <a:schemeClr val="lt1">
-                    <a:lumMod val="95000"/>
-                  </a:schemeClr>
-                </a:solidFill>
-                <a:effectLst>
-                  <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
-                    <a:prstClr val="black">
-                      <a:alpha val="40000"/>
-                    </a:prstClr>
-                  </a:outerShdw>
-                </a:effectLst>
-                <a:latin typeface="+mn-lt"/>
-                <a:ea typeface="+mn-ea"/>
-                <a:cs typeface="+mn-cs"/>
-              </a:defRPr>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US" sz="1600" b="1" i="0" u="none" strike="noStrike" baseline="0">
-                <a:effectLst>
-                  <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
-                    <a:prstClr val="black">
-                      <a:alpha val="40000"/>
-                    </a:prstClr>
-                  </a:outerShdw>
-                </a:effectLst>
-              </a:rPr>
+              <a:rPr lang="en-US" sz="2000"/>
               <a:t>Project NPV Sensitivity to Student Adoption Across Annual Fee Scenarios</a:t>
             </a:r>
           </a:p>
@@ -2672,19 +1808,10 @@
         <a:lstStyle/>
         <a:p>
           <a:pPr>
-            <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" spc="100" baseline="0">
+            <a:defRPr sz="2000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="lt1">
-                  <a:lumMod val="95000"/>
-                </a:schemeClr>
+                <a:schemeClr val="tx2"/>
               </a:solidFill>
-              <a:effectLst>
-                <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
-                  <a:prstClr val="black">
-                    <a:alpha val="40000"/>
-                  </a:prstClr>
-                </a:outerShdw>
-              </a:effectLst>
               <a:latin typeface="+mn-lt"/>
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
@@ -2715,19 +1842,13 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:ln w="34925" cap="rnd">
+            <a:ln w="31750" cap="rnd">
               <a:solidFill>
                 <a:schemeClr val="accent1"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
-            <a:effectLst>
-              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="63000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
+            <a:effectLst/>
           </c:spPr>
           <c:marker>
             <c:symbol val="none"/>
@@ -2838,19 +1959,13 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:ln w="34925" cap="rnd">
+            <a:ln w="31750" cap="rnd">
               <a:solidFill>
                 <a:schemeClr val="accent2"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
-            <a:effectLst>
-              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="63000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
+            <a:effectLst/>
           </c:spPr>
           <c:marker>
             <c:symbol val="none"/>
@@ -2961,19 +2076,13 @@
             </c:strRef>
           </c:tx>
           <c:spPr>
-            <a:ln w="34925" cap="rnd">
+            <a:ln w="31750" cap="rnd">
               <a:solidFill>
                 <a:schemeClr val="accent3"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
-            <a:effectLst>
-              <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-                <a:srgbClr val="000000">
-                  <a:alpha val="63000"/>
-                </a:srgbClr>
-              </a:outerShdw>
-            </a:effectLst>
+            <a:effectLst/>
           </c:spPr>
           <c:marker>
             <c:symbol val="none"/>
@@ -3095,11 +2204,9 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="2000" b="1" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
+                  <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
-                      <a:schemeClr val="lt1">
-                        <a:lumMod val="85000"/>
-                      </a:schemeClr>
+                      <a:schemeClr val="tx2"/>
                     </a:solidFill>
                     <a:latin typeface="+mn-lt"/>
                     <a:ea typeface="+mn-ea"/>
@@ -3107,12 +2214,8 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:rPr lang="en-US" sz="2000"/>
-                  <a:t>Average</a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="en-US" sz="2000" baseline="0"/>
-                  <a:t> (On Campus) Student Adoption Percentage</a:t>
+                  <a:rPr lang="en-US" sz="1600"/>
+                  <a:t>Average (On Campus) Student Adoption Percentage</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -3130,11 +2233,9 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="2000" b="1" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
+                <a:defRPr sz="1600" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
-                    <a:schemeClr val="lt1">
-                      <a:lumMod val="85000"/>
-                    </a:schemeClr>
+                    <a:schemeClr val="tx2"/>
                   </a:solidFill>
                   <a:latin typeface="+mn-lt"/>
                   <a:ea typeface="+mn-ea"/>
@@ -3146,16 +2247,16 @@
           </c:txPr>
         </c:title>
         <c:numFmt formatCode="0.00%" sourceLinked="1"/>
-        <c:majorTickMark val="none"/>
+        <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
         <c:spPr>
           <a:noFill/>
           <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
             <a:solidFill>
-              <a:schemeClr val="lt1">
-                <a:lumMod val="95000"/>
-                <a:alpha val="10000"/>
+              <a:schemeClr val="tx2">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
               </a:schemeClr>
             </a:solidFill>
             <a:round/>
@@ -3169,9 +2270,7 @@
             <a:pPr>
               <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="lt1">
-                    <a:lumMod val="85000"/>
-                  </a:schemeClr>
+                  <a:schemeClr val="tx2"/>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
                 <a:ea typeface="+mn-ea"/>
@@ -3199,9 +2298,9 @@
           <c:spPr>
             <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
               <a:solidFill>
-                <a:schemeClr val="lt1">
-                  <a:lumMod val="95000"/>
-                  <a:alpha val="10000"/>
+                <a:schemeClr val="tx2">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
                 </a:schemeClr>
               </a:solidFill>
               <a:round/>
@@ -3216,11 +2315,9 @@
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
-                  <a:defRPr sz="2000" b="1" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
+                  <a:defRPr sz="2000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                     <a:solidFill>
-                      <a:schemeClr val="lt1">
-                        <a:lumMod val="85000"/>
-                      </a:schemeClr>
+                      <a:schemeClr val="tx2"/>
                     </a:solidFill>
                     <a:latin typeface="+mn-lt"/>
                     <a:ea typeface="+mn-ea"/>
@@ -3229,11 +2326,7 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr lang="en-US" sz="2000"/>
-                  <a:t>5</a:t>
-                </a:r>
-                <a:r>
-                  <a:rPr lang="en-US" sz="2000" baseline="0"/>
-                  <a:t> year Project NPV</a:t>
+                  <a:t>5 year Project NPV</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -3251,11 +2344,9 @@
             <a:lstStyle/>
             <a:p>
               <a:pPr>
-                <a:defRPr sz="2000" b="1" i="0" u="none" strike="noStrike" kern="1200" cap="all" baseline="0">
+                <a:defRPr sz="2000" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                   <a:solidFill>
-                    <a:schemeClr val="lt1">
-                      <a:lumMod val="85000"/>
-                    </a:schemeClr>
+                    <a:schemeClr val="tx2"/>
                   </a:solidFill>
                   <a:latin typeface="+mn-lt"/>
                   <a:ea typeface="+mn-ea"/>
@@ -3284,9 +2375,7 @@
             <a:pPr>
               <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="lt1">
-                    <a:lumMod val="85000"/>
-                  </a:schemeClr>
+                  <a:schemeClr val="tx2"/>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
                 <a:ea typeface="+mn-ea"/>
@@ -3325,9 +2414,7 @@
           <a:pPr>
             <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="lt1">
-                  <a:lumMod val="85000"/>
-                </a:schemeClr>
+                <a:schemeClr val="tx2"/>
               </a:solidFill>
               <a:latin typeface="+mn-lt"/>
               <a:ea typeface="+mn-ea"/>
@@ -3350,28 +2437,17 @@
     </c:extLst>
   </c:chart>
   <c:spPr>
-    <a:gradFill flip="none" rotWithShape="1">
-      <a:gsLst>
-        <a:gs pos="0">
-          <a:schemeClr val="dk1">
-            <a:lumMod val="65000"/>
-            <a:lumOff val="35000"/>
-          </a:schemeClr>
-        </a:gs>
-        <a:gs pos="100000">
-          <a:schemeClr val="dk1">
-            <a:lumMod val="85000"/>
-            <a:lumOff val="15000"/>
-          </a:schemeClr>
-        </a:gs>
-      </a:gsLst>
-      <a:path path="circle">
-        <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-      </a:path>
-      <a:tileRect/>
-    </a:gradFill>
-    <a:ln>
-      <a:noFill/>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx2">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
     </a:ln>
     <a:effectLst/>
   </c:spPr>
@@ -3433,56 +2509,14 @@
 </cs:colorStyle>
 </file>
 
-<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
-  <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
-</cs:colorStyle>
-</file>
-
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="236">
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="231">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="75000"/>
-      </a:schemeClr>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
     <cs:defRPr sz="900" b="1" kern="1200"/>
   </cs:axisTitle>
@@ -3491,29 +2525,35 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="75000"/>
-      </a:schemeClr>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:categoryAxis>
-  <cs:chartArea>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
     <cs:lnRef idx="0"/>
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
-        </a:schemeClr>
+        <a:schemeClr val="bg1"/>
       </a:solidFill>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="dk1">
+          <a:schemeClr val="tx2">
             <a:lumMod val="15000"/>
             <a:lumOff val="85000"/>
           </a:schemeClr>
@@ -3528,9 +2568,7 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="75000"/>
-      </a:schemeClr>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:dataLabel>
@@ -3539,18 +2577,22 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="15000"/>
-        <a:lumOff val="85000"/>
+      <a:schemeClr val="dk2">
+        <a:lumMod val="75000"/>
       </a:schemeClr>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="65000"/>
-          <a:lumOff val="35000"/>
-        </a:schemeClr>
+        <a:schemeClr val="lt1"/>
       </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
     </cs:spPr>
     <cs:defRPr sz="900" kern="1200"/>
     <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
@@ -3558,131 +2600,70 @@
     </cs:bodyPr>
   </cs:dataLabelCallout>
   <cs:dataPoint>
-    <cs:lnRef idx="0">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="3">
       <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:effectRef>
+    </cs:fillRef>
+    <cs:effectRef idx="2"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:miter lim="800000"/>
-      </a:ln>
-      <a:effectLst>
-        <a:glow rad="63500">
-          <a:schemeClr val="phClr">
-            <a:satMod val="175000"/>
-            <a:alpha val="25000"/>
-          </a:schemeClr>
-        </a:glow>
-      </a:effectLst>
-    </cs:spPr>
   </cs:dataPoint>
   <cs:dataPoint3D>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="3">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
-    <cs:effectRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:effectRef>
+    <cs:effectRef idx="2"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:miter lim="800000"/>
-      </a:ln>
-      <a:effectLst>
-        <a:glow rad="63500">
-          <a:schemeClr val="phClr">
-            <a:satMod val="175000"/>
-            <a:alpha val="25000"/>
-          </a:schemeClr>
-        </a:glow>
-      </a:effectLst>
-    </cs:spPr>
   </cs:dataPoint3D>
   <cs:dataPointLine>
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:effectRef>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="2"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="22225" cap="rnd">
+      <a:ln w="31750" cap="rnd">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
+        <a:round/>
       </a:ln>
-      <a:effectLst>
-        <a:glow rad="139700">
-          <a:schemeClr val="phClr">
-            <a:satMod val="175000"/>
-            <a:alpha val="14000"/>
-          </a:schemeClr>
-        </a:glow>
-      </a:effectLst>
     </cs:spPr>
   </cs:dataPointLine>
   <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="3">
       <cs:styleClr val="auto"/>
     </cs:fillRef>
-    <cs:effectRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:effectRef>
+    <cs:effectRef idx="2"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="phClr">
-          <a:lumMod val="60000"/>
-          <a:lumOff val="40000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:effectLst>
-        <a:glow rad="63500">
-          <a:schemeClr val="phClr">
-            <a:satMod val="175000"/>
-            <a:alpha val="25000"/>
-          </a:schemeClr>
-        </a:glow>
-      </a:effectLst>
+      <a:ln w="12700">
+        <a:solidFill>
+          <a:schemeClr val="lt2"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
     </cs:spPr>
   </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="4"/>
+  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
   <cs:dataPointWireframe>
     <cs:lnRef idx="0">
       <cs:styleClr val="auto"/>
     </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
+    <cs:fillRef idx="3"/>
+    <cs:effectRef idx="2"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="rnd">
@@ -3698,16 +2679,14 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="75000"/>
-      </a:schemeClr>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="50000"/>
-            <a:lumOff val="50000"/>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
       </a:ln>
@@ -3719,22 +2698,22 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
+      <a:schemeClr val="dk1"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
         <a:schemeClr val="dk1">
-          <a:lumMod val="50000"/>
-          <a:lumOff val="50000"/>
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
         </a:schemeClr>
       </a:solidFill>
       <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="75000"/>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
       </a:ln>
     </cs:spPr>
   </cs:downBar>
@@ -3743,16 +2722,17 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="50000"/>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="60000"/>
+            <a:lumOff val="40000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
+        <a:prstDash val="dash"/>
       </a:ln>
     </cs:spPr>
   </cs:dropLine>
@@ -3761,13 +2741,13 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="50000"/>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="75000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -3779,7 +2759,7 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
   </cs:floor>
   <cs:gridlineMajor>
@@ -3787,518 +2767,14 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="100000">
-              <a:schemeClr val="dk1">
-                <a:lumMod val="75000"/>
-                <a:lumOff val="25000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="0">
-              <a:schemeClr val="dk1">
-                <a:lumMod val="65000"/>
-                <a:lumOff val="35000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMajor>
-  <cs:gridlineMinor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:gradFill>
-          <a:gsLst>
-            <a:gs pos="100000">
-              <a:schemeClr val="dk1">
-                <a:lumMod val="75000"/>
-                <a:lumOff val="25000"/>
-                <a:alpha val="25000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="0">
-              <a:schemeClr val="dk1">
-                <a:lumMod val="65000"/>
-                <a:lumOff val="35000"/>
-                <a:alpha val="25000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
-        </a:gradFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:gridlineMinor>
-  <cs:hiLoLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:hiLoLine>
-  <cs:leaderLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:leaderLine>
-  <cs:legend>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="75000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:legend>
-  <cs:plotArea>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:plotArea>
-  <cs:plotArea3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:plotArea3D>
-  <cs:seriesAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="75000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:seriesAxis>
-  <cs:seriesLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:seriesLine>
-  <cs:title>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="1400" b="1" kern="1200" cap="none" baseline="0"/>
-  </cs:title>
-  <cs:trendline>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="25400" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:alpha val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:trendline>
-  <cs:trendlineLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="75000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:trendlineLabel>
-  <cs:upBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1">
-          <a:lumMod val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="dk1">
-            <a:lumMod val="50000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:upBar>
-  <cs:valueAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="75000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:valueAxis>
-  <cs:wall>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-  </cs:wall>
-</cs:chartStyle>
-</file>
-
-<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="233">
-  <cs:axisTitle>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" b="1" kern="1200" cap="all"/>
-  </cs:axisTitle>
-  <cs:categoryAxis>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
-      </a:schemeClr>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="10000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:categoryAxis>
-  <cs:chartArea>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:gradFill flip="none" rotWithShape="1">
-        <a:gsLst>
-          <a:gs pos="0">
-            <a:schemeClr val="dk1">
-              <a:lumMod val="65000"/>
-              <a:lumOff val="35000"/>
-            </a:schemeClr>
-          </a:gs>
-          <a:gs pos="100000">
-            <a:schemeClr val="dk1">
-              <a:lumMod val="85000"/>
-              <a:lumOff val="15000"/>
-            </a:schemeClr>
-          </a:gs>
-        </a:gsLst>
-        <a:path path="circle">
-          <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-        </a:path>
-        <a:tileRect/>
-      </a:gradFill>
-    </cs:spPr>
-    <cs:defRPr sz="1000" kern="1200"/>
-  </cs:chartArea>
-  <cs:dataLabel>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataLabel>
-  <cs:dataLabelCallout>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="dk1">
-        <a:lumMod val="65000"/>
-        <a:lumOff val="35000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="lt1"/>
-      </a:solidFill>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
-      <a:spAutoFit/>
-    </cs:bodyPr>
-  </cs:dataLabelCallout>
-  <cs:dataPoint>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="3">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="3"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint>
-  <cs:dataPoint3D>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="3">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="3"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:dataPoint3D>
-  <cs:dataPointLine>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="3"/>
-    <cs:effectRef idx="3"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="34925" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointLine>
-  <cs:dataPointMarker>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="3">
-      <cs:styleClr val="auto"/>
-    </cs:fillRef>
-    <cs:effectRef idx="3"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointMarker>
-  <cs:dataPointMarkerLayout symbol="circle" size="6"/>
-  <cs:dataPointWireframe>
-    <cs:lnRef idx="0">
-      <cs:styleClr val="auto"/>
-    </cs:lnRef>
-    <cs:fillRef idx="3"/>
-    <cs:effectRef idx="3"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="rnd">
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dataPointWireframe>
-  <cs:dataTable>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
-      </a:schemeClr>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-    <cs:defRPr sz="900" kern="1200"/>
-  </cs:dataTable>
-  <cs:downBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:solidFill>
-        <a:schemeClr val="dk1">
-          <a:lumMod val="75000"/>
-          <a:lumOff val="25000"/>
-        </a:schemeClr>
-      </a:solidFill>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </a:ln>
-    </cs:spPr>
-  </cs:downBar>
-  <cs:dropLine>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:prstDash val="dash"/>
-      </a:ln>
-    </cs:spPr>
-  </cs:dropLine>
-  <cs:errorBar>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:round/>
-      </a:ln>
-    </cs:spPr>
-  </cs:errorBar>
-  <cs:floor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-  </cs:floor>
-  <cs:gridlineMajor>
-    <cs:lnRef idx="0"/>
-    <cs:fillRef idx="0"/>
-    <cs:effectRef idx="0"/>
-    <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
-    </cs:fontRef>
-    <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-        <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="10000"/>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -4310,14 +2786,14 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln>
         <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="5000"/>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
           </a:schemeClr>
         </a:solidFill>
       </a:ln>
@@ -4328,14 +2804,14 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="60000"/>
+            <a:lumOff val="40000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:prstDash val="dash"/>
@@ -4347,14 +2823,14 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
           </a:schemeClr>
         </a:solidFill>
       </a:ln>
@@ -4365,9 +2841,7 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
-      </a:schemeClr>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:legend>
@@ -4376,7 +2850,7 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
   </cs:plotArea>
   <cs:plotArea3D>
@@ -4384,7 +2858,7 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
   </cs:plotArea3D>
   <cs:seriesAxis>
@@ -4392,16 +2866,14 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
-      </a:schemeClr>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
         <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
         <a:round/>
@@ -4414,17 +2886,17 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1"/>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
     <cs:spPr>
-      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
+          <a:schemeClr val="tx2">
+            <a:lumMod val="60000"/>
+            <a:lumOff val="40000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:round/>
+        <a:prstDash val="dash"/>
       </a:ln>
     </cs:spPr>
   </cs:seriesLine>
@@ -4433,19 +2905,9 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="95000"/>
-      </a:schemeClr>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
-    <cs:defRPr sz="1600" b="1" kern="1200" spc="100" baseline="0">
-      <a:effectLst>
-        <a:outerShdw blurRad="50800" dist="38100" dir="5400000" algn="t" rotWithShape="0">
-          <a:prstClr val="black">
-            <a:alpha val="40000"/>
-          </a:prstClr>
-        </a:outerShdw>
-      </a:effectLst>
-    </cs:defRPr>
+    <cs:defRPr sz="1600" b="1" kern="1200"/>
   </cs:title>
   <cs:trendline>
     <cs:lnRef idx="0">
@@ -4454,13 +2916,14 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
     <cs:spPr>
       <a:ln w="19050" cap="rnd">
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
+        <a:prstDash val="sysDash"/>
       </a:ln>
     </cs:spPr>
   </cs:trendline>
@@ -4469,9 +2932,7 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
-      </a:schemeClr>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:trendlineLabel>
@@ -4480,7 +2941,7 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
     <cs:spPr>
       <a:solidFill>
@@ -4488,9 +2949,9 @@
       </a:solidFill>
       <a:ln w="9525">
         <a:solidFill>
-          <a:schemeClr val="lt1">
-            <a:lumMod val="95000"/>
-            <a:alpha val="54000"/>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
           </a:schemeClr>
         </a:solidFill>
       </a:ln>
@@ -4501,9 +2962,7 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="lt1">
-        <a:lumMod val="85000"/>
-      </a:schemeClr>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
     <cs:defRPr sz="900" kern="1200"/>
   </cs:valueAxis>
@@ -4512,54 +2971,13 @@
     <cs:fillRef idx="0"/>
     <cs:effectRef idx="0"/>
     <cs:fontRef idx="minor">
-      <a:schemeClr val="tx1"/>
+      <a:schemeClr val="tx2"/>
     </cs:fontRef>
   </cs:wall>
 </cs:chartStyle>
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>1178790</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>37013</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>33</xdr:col>
-      <xdr:colOff>168870</xdr:colOff>
-      <xdr:row>64</xdr:row>
-      <xdr:rowOff>123597</xdr:rowOff>
-    </xdr:to>
-    <xdr:graphicFrame macro="">
-      <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="Chart 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{BC03EC98-F8D4-4F5C-3834-F2092621E320}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGraphicFramePr/>
-      </xdr:nvGraphicFramePr>
-      <xdr:xfrm>
-        <a:off x="0" y="0"/>
-        <a:ext cx="0" cy="0"/>
-      </xdr:xfrm>
-      <a:graphic>
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </xdr:graphicFrame>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -4941,14 +3359,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="122" t="s">
+      <c r="B2" s="130" t="s">
         <v>61</v>
       </c>
-      <c r="C2" s="123"/>
-      <c r="E2" s="124" t="s">
+      <c r="C2" s="131"/>
+      <c r="E2" s="132" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="125"/>
+      <c r="F2" s="133"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B3" s="3" t="s">
@@ -4989,10 +3407,10 @@
       </c>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B6" s="126" t="s">
+      <c r="B6" s="134" t="s">
         <v>60</v>
       </c>
-      <c r="C6" s="126"/>
+      <c r="C6" s="134"/>
       <c r="E6" s="96" t="s">
         <v>122</v>
       </c>
@@ -5030,13 +3448,13 @@
       <c r="C9" s="3">
         <v>18</v>
       </c>
-      <c r="E9" s="127" t="s">
+      <c r="E9" s="135" t="s">
         <v>157</v>
       </c>
-      <c r="F9" s="128"/>
-      <c r="G9" s="128"/>
-      <c r="H9" s="128"/>
-      <c r="I9" s="129"/>
+      <c r="F9" s="136"/>
+      <c r="G9" s="136"/>
+      <c r="H9" s="136"/>
+      <c r="I9" s="137"/>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B10" s="3" t="s">
@@ -5106,10 +3524,10 @@
       </c>
     </row>
     <row r="13" spans="2:9" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="130" t="s">
+      <c r="B13" s="138" t="s">
         <v>69</v>
       </c>
-      <c r="C13" s="131"/>
+      <c r="C13" s="139"/>
       <c r="E13" s="56" t="s">
         <v>100</v>
       </c>
@@ -5226,10 +3644,10 @@
       </c>
     </row>
     <row r="19" spans="2:9" ht="16" x14ac:dyDescent="0.2">
-      <c r="B19" s="132" t="s">
+      <c r="B19" s="140" t="s">
         <v>68</v>
       </c>
-      <c r="C19" s="123"/>
+      <c r="C19" s="131"/>
     </row>
     <row r="20" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B20" s="3" t="s">
@@ -5276,10 +3694,10 @@
       <c r="C25" s="48"/>
     </row>
     <row r="26" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B26" s="126" t="s">
+      <c r="B26" s="134" t="s">
         <v>74</v>
       </c>
-      <c r="C26" s="126"/>
+      <c r="C26" s="134"/>
     </row>
     <row r="27" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B27" s="1" t="s">
@@ -5330,10 +3748,10 @@
       </c>
     </row>
     <row r="34" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B34" s="126" t="s">
+      <c r="B34" s="134" t="s">
         <v>185</v>
       </c>
-      <c r="C34" s="126"/>
+      <c r="C34" s="134"/>
     </row>
     <row r="35" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B35" s="3" t="s">
@@ -5352,10 +3770,10 @@
       </c>
     </row>
     <row r="38" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B38" s="126" t="s">
+      <c r="B38" s="134" t="s">
         <v>78</v>
       </c>
-      <c r="C38" s="126"/>
+      <c r="C38" s="134"/>
     </row>
     <row r="39" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B39" s="1" t="s">
@@ -5406,10 +3824,10 @@
       </c>
     </row>
     <row r="46" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B46" s="126" t="s">
+      <c r="B46" s="134" t="s">
         <v>190</v>
       </c>
-      <c r="C46" s="126"/>
+      <c r="C46" s="134"/>
     </row>
     <row r="47" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B47" s="1" t="s">
@@ -5466,24 +3884,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:26" x14ac:dyDescent="0.2">
-      <c r="M1" s="139" t="s">
+      <c r="M1" s="147" t="s">
         <v>53</v>
       </c>
-      <c r="N1" s="139"/>
-      <c r="O1" s="139"/>
-      <c r="P1" s="139"/>
+      <c r="N1" s="147"/>
+      <c r="O1" s="147"/>
+      <c r="P1" s="147"/>
     </row>
     <row r="2" spans="2:26" x14ac:dyDescent="0.2">
-      <c r="B2" s="137" t="s">
+      <c r="B2" s="145" t="s">
         <v>24</v>
       </c>
-      <c r="C2" s="138"/>
-      <c r="E2" s="140" t="s">
+      <c r="C2" s="146"/>
+      <c r="E2" s="148" t="s">
         <v>124</v>
       </c>
-      <c r="F2" s="141"/>
-      <c r="G2" s="141"/>
-      <c r="H2" s="142"/>
+      <c r="F2" s="149"/>
+      <c r="G2" s="149"/>
+      <c r="H2" s="150"/>
       <c r="M2" s="39" t="s">
         <v>40</v>
       </c>
@@ -5863,13 +4281,13 @@
         <v>21</v>
       </c>
       <c r="C13" s="23"/>
-      <c r="E13" s="161" t="s">
+      <c r="E13" s="151" t="s">
         <v>125</v>
       </c>
-      <c r="F13" s="161"/>
-      <c r="G13" s="161"/>
-      <c r="H13" s="161"/>
-      <c r="I13" s="164"/>
+      <c r="F13" s="151"/>
+      <c r="G13" s="151"/>
+      <c r="H13" s="151"/>
+      <c r="I13" s="10"/>
       <c r="L13" s="34"/>
     </row>
     <row r="14" spans="2:26" x14ac:dyDescent="0.2">
@@ -5879,16 +4297,15 @@
       <c r="C14" s="6">
         <v>39.799999999999997</v>
       </c>
-      <c r="E14" s="162" t="s">
+      <c r="E14" s="152" t="s">
         <v>207</v>
       </c>
-      <c r="F14" s="162"/>
-      <c r="G14" s="163">
+      <c r="F14" s="152"/>
+      <c r="G14" s="155">
         <f>Usability!I4*12</f>
         <v>124629.04109589041</v>
       </c>
-      <c r="H14" s="163"/>
-      <c r="I14" s="158"/>
+      <c r="H14" s="155"/>
       <c r="L14" s="34"/>
     </row>
     <row r="15" spans="2:26" x14ac:dyDescent="0.2">
@@ -6019,10 +4436,10 @@
       </c>
     </row>
     <row r="21" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B21" s="135" t="s">
+      <c r="B21" s="143" t="s">
         <v>158</v>
       </c>
-      <c r="C21" s="136"/>
+      <c r="C21" s="144"/>
       <c r="E21" s="25" t="s">
         <v>28</v>
       </c>
@@ -6046,10 +4463,10 @@
       <c r="C22" s="3">
         <v>2</v>
       </c>
-      <c r="E22" s="159" t="s">
+      <c r="E22" s="153" t="s">
         <v>206</v>
       </c>
-      <c r="F22" s="160"/>
+      <c r="F22" s="154"/>
     </row>
     <row r="23" spans="2:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B23" s="16" t="s">
@@ -6058,10 +4475,10 @@
       <c r="C23" s="17">
         <v>40000</v>
       </c>
-      <c r="F23" s="133" t="s">
+      <c r="F23" s="141" t="s">
         <v>173</v>
       </c>
-      <c r="G23" s="134"/>
+      <c r="G23" s="142"/>
     </row>
     <row r="24" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B24" s="16" t="s">
@@ -6171,10 +4588,10 @@
       <c r="E2" s="104" t="s">
         <v>195</v>
       </c>
-      <c r="H2" s="121" t="s">
+      <c r="H2" s="156" t="s">
         <v>152</v>
       </c>
-      <c r="I2" s="121"/>
+      <c r="I2" s="156"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B3" s="91" t="s">
@@ -6511,16 +4928,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A1" s="145" t="s">
+      <c r="A1" s="157" t="s">
         <v>180</v>
       </c>
-      <c r="B1" s="145"/>
-      <c r="C1" s="145"/>
-      <c r="D1" s="145"/>
-      <c r="E1" s="145"/>
-      <c r="F1" s="145"/>
-      <c r="G1" s="145"/>
-      <c r="H1" s="145"/>
+      <c r="B1" s="157"/>
+      <c r="C1" s="157"/>
+      <c r="D1" s="157"/>
+      <c r="E1" s="157"/>
+      <c r="F1" s="157"/>
+      <c r="G1" s="157"/>
+      <c r="H1" s="157"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
@@ -6863,16 +5280,16 @@
       <c r="D15" s="83"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A16" s="145" t="s">
+      <c r="A16" s="157" t="s">
         <v>179</v>
       </c>
-      <c r="B16" s="145"/>
-      <c r="C16" s="145"/>
-      <c r="D16" s="145"/>
-      <c r="E16" s="145"/>
-      <c r="F16" s="145"/>
-      <c r="G16" s="145"/>
-      <c r="H16" s="145"/>
+      <c r="B16" s="157"/>
+      <c r="C16" s="157"/>
+      <c r="D16" s="157"/>
+      <c r="E16" s="157"/>
+      <c r="F16" s="157"/>
+      <c r="G16" s="157"/>
+      <c r="H16" s="157"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
@@ -7116,25 +5533,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B1" s="146" t="s">
+      <c r="B1" s="158" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="146"/>
+      <c r="C1" s="158"/>
       <c r="F1" s="9"/>
-      <c r="G1" s="147" t="s">
+      <c r="G1" s="159" t="s">
         <v>12</v>
       </c>
-      <c r="H1" s="148"/>
+      <c r="H1" s="160"/>
       <c r="I1" s="10"/>
-      <c r="J1" s="147" t="s">
+      <c r="J1" s="159" t="s">
         <v>120</v>
       </c>
-      <c r="K1" s="148"/>
+      <c r="K1" s="160"/>
       <c r="L1" s="10"/>
-      <c r="M1" s="147" t="s">
+      <c r="M1" s="159" t="s">
         <v>13</v>
       </c>
-      <c r="N1" s="148"/>
+      <c r="N1" s="160"/>
     </row>
     <row r="2" spans="2:14" x14ac:dyDescent="0.2">
       <c r="B2" s="3" t="s">
@@ -7484,12 +5901,12 @@
       </c>
     </row>
     <row r="14" spans="2:14" x14ac:dyDescent="0.2">
-      <c r="B14" s="149" t="s">
+      <c r="B14" s="161" t="s">
         <v>119</v>
       </c>
-      <c r="C14" s="150"/>
-      <c r="D14" s="150"/>
-      <c r="E14" s="150"/>
+      <c r="C14" s="162"/>
+      <c r="D14" s="162"/>
+      <c r="E14" s="162"/>
       <c r="F14" s="8"/>
       <c r="G14" s="1">
         <v>11</v>
@@ -8728,16 +7145,16 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="144" t="s">
+      <c r="B2" s="164" t="s">
         <v>201</v>
       </c>
-      <c r="C2" s="144"/>
-      <c r="D2" s="144"/>
-      <c r="E2" s="144"/>
-      <c r="H2" s="143" t="s">
+      <c r="C2" s="164"/>
+      <c r="D2" s="164"/>
+      <c r="E2" s="164"/>
+      <c r="H2" s="163" t="s">
         <v>203</v>
       </c>
-      <c r="I2" s="143"/>
+      <c r="I2" s="163"/>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.2">
       <c r="B3" s="91" t="s">
@@ -8795,12 +7212,12 @@
       </c>
     </row>
     <row r="6" spans="2:9" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="144" t="s">
+      <c r="B6" s="164" t="s">
         <v>200</v>
       </c>
-      <c r="C6" s="144"/>
-      <c r="D6" s="144"/>
-      <c r="E6" s="144"/>
+      <c r="C6" s="164"/>
+      <c r="D6" s="164"/>
+      <c r="E6" s="164"/>
       <c r="H6" s="1">
         <f t="shared" ref="H6:H8" si="1">1+H5</f>
         <v>3</v>
@@ -8811,10 +7228,10 @@
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B7" s="153" t="s">
+      <c r="B7" s="165" t="s">
         <v>204</v>
       </c>
-      <c r="C7" s="154"/>
+      <c r="C7" s="166"/>
       <c r="D7" s="91" t="s">
         <v>202</v>
       </c>
@@ -8831,11 +7248,11 @@
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.2">
-      <c r="B8" s="155">
+      <c r="B8" s="167">
         <f>Usability!I4*12</f>
         <v>124629.04109589041</v>
       </c>
-      <c r="C8" s="156"/>
+      <c r="C8" s="168"/>
       <c r="D8" s="12">
         <v>0.5</v>
       </c>
@@ -8843,7 +7260,7 @@
         <f>B8*D8</f>
         <v>62314.520547945205</v>
       </c>
-      <c r="H8" s="157">
+      <c r="H8" s="121">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
@@ -8924,7 +7341,7 @@
       <c r="K1" s="113" t="s">
         <v>209</v>
       </c>
-      <c r="L1" s="175" t="s">
+      <c r="L1" s="128" t="s">
         <v>211</v>
       </c>
     </row>
@@ -9070,10 +7487,10 @@
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K4)</f>
         <v>45565.086703934605</v>
       </c>
-      <c r="O4" s="151" t="s">
+      <c r="O4" s="129" t="s">
         <v>184</v>
       </c>
-      <c r="P4" s="151"/>
+      <c r="P4" s="129"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" s="115">
@@ -11934,7 +10351,6 @@
     <mergeCell ref="O4:P4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -11950,41 +10366,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B1" s="139"/>
-      <c r="C1" s="139"/>
+      <c r="B1" s="147"/>
+      <c r="C1" s="147"/>
     </row>
     <row r="2" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="152"/>
       <c r="M2" s="120"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B3" s="173">
+      <c r="B3" s="126">
         <v>0.12</v>
       </c>
-      <c r="C3" s="171" t="s">
+      <c r="C3" s="125" t="s">
         <v>182</v>
       </c>
-      <c r="D3" s="168" t="s">
+      <c r="D3" s="171" t="s">
         <v>208</v>
       </c>
-      <c r="E3" s="166"/>
-      <c r="F3" s="166"/>
-      <c r="G3" s="166"/>
-      <c r="H3" s="166"/>
-      <c r="I3" s="166"/>
-      <c r="J3" s="166"/>
-      <c r="K3" s="166"/>
+      <c r="E3" s="172"/>
+      <c r="F3" s="172"/>
+      <c r="G3" s="172"/>
+      <c r="H3" s="172"/>
+      <c r="I3" s="172"/>
+      <c r="J3" s="172"/>
+      <c r="K3" s="172"/>
     </row>
     <row r="4" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10"/>
-      <c r="B4" s="174">
+      <c r="B4" s="127">
         <v>180</v>
       </c>
-      <c r="C4" s="174">
+      <c r="C4" s="127">
         <f>Cashflow!P5</f>
         <v>185448.79524921341</v>
       </c>
-      <c r="D4" s="169">
+      <c r="D4" s="123">
         <v>180</v>
       </c>
       <c r="E4" s="12">
@@ -12018,10 +10433,10 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" s="10"/>
-      <c r="B5" s="172" t="s">
+      <c r="B5" s="169" t="s">
         <v>196</v>
       </c>
-      <c r="C5" s="170">
+      <c r="C5" s="124">
         <v>0.1</v>
       </c>
       <c r="D5" s="12">
@@ -12052,8 +10467,8 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" s="10"/>
-      <c r="B6" s="165"/>
-      <c r="C6" s="167">
+      <c r="B6" s="170"/>
+      <c r="C6" s="122">
         <f>C5+0.01</f>
         <v>0.11</v>
       </c>
@@ -12084,8 +10499,8 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" s="10"/>
-      <c r="B7" s="165"/>
-      <c r="C7" s="167">
+      <c r="B7" s="170"/>
+      <c r="C7" s="122">
         <f t="shared" ref="C7:C15" si="1">C6+0.01</f>
         <v>0.12</v>
       </c>
@@ -12116,8 +10531,8 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" s="10"/>
-      <c r="B8" s="165"/>
-      <c r="C8" s="167">
+      <c r="B8" s="170"/>
+      <c r="C8" s="122">
         <f t="shared" si="1"/>
         <v>0.13</v>
       </c>
@@ -12148,8 +10563,8 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" s="10"/>
-      <c r="B9" s="165"/>
-      <c r="C9" s="167">
+      <c r="B9" s="170"/>
+      <c r="C9" s="122">
         <f t="shared" si="1"/>
         <v>0.14000000000000001</v>
       </c>
@@ -12179,8 +10594,8 @@
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B10" s="165"/>
-      <c r="C10" s="167">
+      <c r="B10" s="170"/>
+      <c r="C10" s="122">
         <f t="shared" si="1"/>
         <v>0.15000000000000002</v>
       </c>
@@ -12210,8 +10625,8 @@
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B11" s="165"/>
-      <c r="C11" s="167">
+      <c r="B11" s="170"/>
+      <c r="C11" s="122">
         <f t="shared" si="1"/>
         <v>0.16000000000000003</v>
       </c>
@@ -12241,8 +10656,8 @@
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B12" s="165"/>
-      <c r="C12" s="167">
+      <c r="B12" s="170"/>
+      <c r="C12" s="122">
         <f t="shared" si="1"/>
         <v>0.17000000000000004</v>
       </c>
@@ -12272,8 +10687,8 @@
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B13" s="165"/>
-      <c r="C13" s="167">
+      <c r="B13" s="170"/>
+      <c r="C13" s="122">
         <f t="shared" si="1"/>
         <v>0.18000000000000005</v>
       </c>
@@ -12303,8 +10718,8 @@
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B14" s="165"/>
-      <c r="C14" s="167">
+      <c r="B14" s="170"/>
+      <c r="C14" s="122">
         <f t="shared" si="1"/>
         <v>0.19000000000000006</v>
       </c>
@@ -12334,8 +10749,8 @@
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B15" s="165"/>
-      <c r="C15" s="167">
+      <c r="B15" s="170"/>
+      <c r="C15" s="122">
         <f t="shared" si="1"/>
         <v>0.20000000000000007</v>
       </c>
@@ -12386,6 +10801,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="d4398b65-27a0-431f-bb10-646010ce6561" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A4B588CF2F739442BBACEEFB9E32E115" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="bd739693acba30017d398d9f3cc91eb1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="d4398b65-27a0-431f-bb10-646010ce6561" xmlns:ns4="1926e0f5-0cc0-4557-b4d7-f87d799596a8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d9455580dc58f441b43481b9dfd0cb15" ns3:_="" ns4:_="">
     <xsd:import namespace="d4398b65-27a0-431f-bb10-646010ce6561"/>
@@ -12612,24 +11044,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{04AAADC4-082E-4732-B6C6-8AD62649A126}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="1926e0f5-0cc0-4557-b4d7-f87d799596a8"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="d4398b65-27a0-431f-bb10-646010ce6561"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="d4398b65-27a0-431f-bb10-646010ce6561" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2E1AF55F-D374-449E-AE21-16FF33F48129}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E0E3D0C8-3787-4A9D-80DE-BA4853E488D3}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -12646,29 +11086,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2E1AF55F-D374-449E-AE21-16FF33F48129}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{04AAADC4-082E-4732-B6C6-8AD62649A126}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="1926e0f5-0cc0-4557-b4d7-f87d799596a8"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="d4398b65-27a0-431f-bb10-646010ce6561"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Update Scooter Fleet page with new Annual Discounted Cashflow chart, master systems table, and group attribution
</commit_message>
<xml_diff>
--- a/Electic Scooter Fleet/INDE 460 - Cost Final Project.xlsx
+++ b/Electic Scooter Fleet/INDE 460 - Cost Final Project.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/evdawgsmac/LocalFiles/P_Path/Job Search/Project Portfolio/Electic Scooter Fleet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2C356E1-FBD8-8F40-A7B3-15F8E1037979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{411DF8F8-D5B4-9C46-A600-3D4547F60252}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17500" activeTab="8" xr2:uid="{4E1F7FCE-C5AE-4A76-87F8-0DC26954148D}"/>
+    <workbookView xWindow="-3180" yWindow="-21000" windowWidth="40560" windowHeight="21000" activeTab="7" xr2:uid="{4E1F7FCE-C5AE-4A76-87F8-0DC26954148D}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Details" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,8 @@
     <sheet name="CR Finance Options" sheetId="7" r:id="rId6"/>
     <sheet name="Revenue" sheetId="9" r:id="rId7"/>
     <sheet name="Cashflow" sheetId="3" r:id="rId8"/>
-    <sheet name="PROJECT ANALYSIS" sheetId="11" r:id="rId9"/>
+    <sheet name="Annual Cashflow" sheetId="12" r:id="rId9"/>
+    <sheet name="PROJECT ANALYSIS" sheetId="11" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="293" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="217">
   <si>
     <t>Cost</t>
   </si>
@@ -702,12 +703,27 @@
   <si>
     <t>Discounted Project Value</t>
   </si>
+  <si>
+    <t>Annual Revenue</t>
+  </si>
+  <si>
+    <t>Annual Costs</t>
+  </si>
+  <si>
+    <t>Cumulative NPV</t>
+  </si>
+  <si>
+    <t>Discounted Outflow</t>
+  </si>
+  <si>
+    <t>Discounted Inflow</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="8">
+  <numFmts count="9">
     <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00_);[Red]\(&quot;$&quot;#,##0.00\)"/>
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
@@ -716,6 +732,7 @@
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
     <numFmt numFmtId="168" formatCode="0.000"/>
+    <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0.00;[Red]&quot;$&quot;#,##0.00"/>
   </numFmts>
   <fonts count="13" x14ac:knownFonts="1">
     <font>
@@ -1297,7 +1314,7 @@
     <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="173">
+  <cellXfs count="175">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1733,6 +1750,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -1759,6 +1778,481 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Annual</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> Discounted Cashflow (8% MARR)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Annual Cashflow'!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Annual Revenue</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:val>
+            <c:numRef>
+              <c:f>'Annual Cashflow'!$B$2:$B$6</c:f>
+              <c:numCache>
+                <c:formatCode>"$"#,##0.00;[Red]"$"#,##0.00</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>210496.63225562812</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>204752.50830366375</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>194415.65583672572</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>184643.24614511634</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>178936.03870423092</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-6D96-274F-A4AE-92E9F2CE80F7}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Annual Cashflow'!$C$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Annual Costs</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:val>
+            <c:numRef>
+              <c:f>'Annual Cashflow'!$C$2:$C$6</c:f>
+              <c:numCache>
+                <c:formatCode>"$"#,##0.00;[Red]"$"#,##0.00</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>249372.7018597956</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>179313.43397986534</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>169520.57810714102</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>104193.67102111128</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>102318.26807857092</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-6D96-274F-A4AE-92E9F2CE80F7}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1883744320"/>
+        <c:axId val="1883746560"/>
+      </c:barChart>
+      <c:lineChart>
+        <c:grouping val="standard"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Annual Cashflow'!$D$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Cumulative NPV</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="28575" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:val>
+            <c:numRef>
+              <c:f>'Annual Cashflow'!$D$2:$D$6</c:f>
+              <c:numCache>
+                <c:formatCode>"$"#,##0.00;[Red]"$"#,##0.00</c:formatCode>
+                <c:ptCount val="5"/>
+                <c:pt idx="0">
+                  <c:v>-38876.069604167482</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>-13436.995280369068</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>11458.082449215639</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>91907.657573220698</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>168525.42819888069</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-6D96-274F-A4AE-92E9F2CE80F7}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:marker val="1"/>
+        <c:smooth val="0"/>
+        <c:axId val="1883744320"/>
+        <c:axId val="1883746560"/>
+      </c:lineChart>
+      <c:catAx>
+        <c:axId val="1883744320"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1883746560"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1883746560"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="&quot;$&quot;#,##0.00;[Red]&quot;$&quot;#,##0.00" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1883744320"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
@@ -1902,37 +2396,37 @@
                 <c:formatCode>"$"#,##0.00</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>67016.123779569025</c:v>
+                  <c:v>52913.317904291755</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>126232.45951439119</c:v>
+                  <c:v>110719.37305158621</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>185448.79524921341</c:v>
+                  <c:v>168525.42819888081</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>244665.13098403567</c:v>
+                  <c:v>226331.48334617523</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>303881.46671885811</c:v>
+                  <c:v>284137.53849346994</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>363097.80245368037</c:v>
+                  <c:v>341943.59364076459</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>422314.13818850258</c:v>
+                  <c:v>399749.64878805896</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>481530.47392332484</c:v>
+                  <c:v>457555.70393535355</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>540746.80965814728</c:v>
+                  <c:v>515361.7590826482</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>599963.1453929696</c:v>
+                  <c:v>573167.81422994286</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>659179.48112779169</c:v>
+                  <c:v>630973.86937723751</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2019,37 +2513,37 @@
                 <c:formatCode>"$"#,##0.00</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>166383.37638373568</c:v>
+                  <c:v>152280.57050845848</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>235536.43737897463</c:v>
+                  <c:v>220023.35091616964</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>304689.49837421346</c:v>
+                  <c:v>287766.13132388081</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>373842.55936945241</c:v>
+                  <c:v>355508.91173159186</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>442995.62036469148</c:v>
+                  <c:v>423251.69213930337</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>512148.68135993078</c:v>
+                  <c:v>490994.47254701483</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>581301.7423551695</c:v>
+                  <c:v>558737.25295472587</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>650454.80335040845</c:v>
+                  <c:v>626480.03336243704</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>719607.86434564739</c:v>
+                  <c:v>694222.81377014844</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>788760.92534088634</c:v>
+                  <c:v>761965.59417785995</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>857913.98633612553</c:v>
+                  <c:v>829708.374585571</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2136,37 +2630,37 @@
                 <c:formatCode>"$"#,##0.00</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>298873.04652262456</c:v>
+                  <c:v>284770.24064734747</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>381275.0745317525</c:v>
+                  <c:v>365761.98806894751</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>463677.10254088021</c:v>
+                  <c:v>446753.73549054749</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>546079.13055000803</c:v>
+                  <c:v>527745.48291214765</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>628481.15855913586</c:v>
+                  <c:v>608737.23033374781</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>710883.18656826427</c:v>
+                  <c:v>689728.9777553482</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>793285.21457739174</c:v>
+                  <c:v>770720.72517694836</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>875687.2425865198</c:v>
+                  <c:v>851712.47259854851</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>958089.27059564739</c:v>
+                  <c:v>932704.22002014832</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1040491.2986047756</c:v>
+                  <c:v>1013695.9674417488</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1122893.3266139037</c:v>
+                  <c:v>1094687.7148633488</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2509,7 +3003,550 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="231">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -2982,6 +4019,47 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>50800</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>158750</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F9EB3E8A-5D85-82D4-BF8A-5A59A3903421}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
       <xdr:colOff>996337</xdr:colOff>
       <xdr:row>17</xdr:row>
       <xdr:rowOff>4386</xdr:rowOff>
@@ -3855,6 +4933,452 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9ECABA95-71D1-0E46-8056-8FE7EC645263}">
+  <dimension ref="A1:M18"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="14.6640625" customWidth="1"/>
+    <col min="2" max="2" width="19.6640625" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" customWidth="1"/>
+    <col min="4" max="11" width="14.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B1" s="147"/>
+      <c r="C1" s="147"/>
+    </row>
+    <row r="2" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="M2" s="120"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B3" s="126">
+        <v>0.12</v>
+      </c>
+      <c r="C3" s="125" t="s">
+        <v>182</v>
+      </c>
+      <c r="D3" s="171" t="s">
+        <v>208</v>
+      </c>
+      <c r="E3" s="172"/>
+      <c r="F3" s="172"/>
+      <c r="G3" s="172"/>
+      <c r="H3" s="172"/>
+      <c r="I3" s="172"/>
+      <c r="J3" s="172"/>
+      <c r="K3" s="172"/>
+    </row>
+    <row r="4" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="10"/>
+      <c r="B4" s="127">
+        <v>180</v>
+      </c>
+      <c r="C4" s="127">
+        <f>Cashflow!R5</f>
+        <v>168525.42819888081</v>
+      </c>
+      <c r="D4" s="123">
+        <v>180</v>
+      </c>
+      <c r="E4" s="12">
+        <f>D4+10</f>
+        <v>190</v>
+      </c>
+      <c r="F4" s="12">
+        <f t="shared" ref="F4:J4" si="0">E4+10</f>
+        <v>200</v>
+      </c>
+      <c r="G4" s="12">
+        <f t="shared" si="0"/>
+        <v>210</v>
+      </c>
+      <c r="H4" s="12">
+        <f t="shared" si="0"/>
+        <v>220</v>
+      </c>
+      <c r="I4" s="12">
+        <f t="shared" si="0"/>
+        <v>230</v>
+      </c>
+      <c r="J4" s="12">
+        <f t="shared" si="0"/>
+        <v>240</v>
+      </c>
+      <c r="K4" s="12">
+        <f>J4+10</f>
+        <v>250</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A5" s="10"/>
+      <c r="B5" s="169" t="s">
+        <v>196</v>
+      </c>
+      <c r="C5" s="124">
+        <v>0.1</v>
+      </c>
+      <c r="D5" s="12">
+        <f t="dataTable" ref="D5:K15" dt2D="1" dtr="1" r1="B4" r2="B3"/>
+        <v>52913.317904291755</v>
+      </c>
+      <c r="E5" s="12">
+        <v>86035.73543901401</v>
+      </c>
+      <c r="F5" s="12">
+        <v>119158.15297373626</v>
+      </c>
+      <c r="G5" s="12">
+        <v>152280.57050845848</v>
+      </c>
+      <c r="H5" s="12">
+        <v>185402.98804318075</v>
+      </c>
+      <c r="I5" s="12">
+        <v>218525.40557790297</v>
+      </c>
+      <c r="J5" s="12">
+        <v>251647.82311262519</v>
+      </c>
+      <c r="K5" s="12">
+        <v>284770.24064734747</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A6" s="10"/>
+      <c r="B6" s="170"/>
+      <c r="C6" s="122">
+        <f>C5+0.01</f>
+        <v>0.11</v>
+      </c>
+      <c r="D6" s="12">
+        <v>110719.37305158621</v>
+      </c>
+      <c r="E6" s="12">
+        <v>147154.03233978077</v>
+      </c>
+      <c r="F6" s="12">
+        <v>183588.6916279752</v>
+      </c>
+      <c r="G6" s="12">
+        <v>220023.35091616964</v>
+      </c>
+      <c r="H6" s="12">
+        <v>256458.01020436408</v>
+      </c>
+      <c r="I6" s="12">
+        <v>292892.66949255858</v>
+      </c>
+      <c r="J6" s="12">
+        <v>329327.32878075307</v>
+      </c>
+      <c r="K6" s="12">
+        <v>365761.98806894751</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A7" s="10"/>
+      <c r="B7" s="170"/>
+      <c r="C7" s="122">
+        <f t="shared" ref="C7:C15" si="1">C6+0.01</f>
+        <v>0.12</v>
+      </c>
+      <c r="D7" s="12">
+        <v>168525.42819888081</v>
+      </c>
+      <c r="E7" s="12">
+        <v>208272.32924054743</v>
+      </c>
+      <c r="F7" s="12">
+        <v>248019.23028221415</v>
+      </c>
+      <c r="G7" s="12">
+        <v>287766.13132388081</v>
+      </c>
+      <c r="H7" s="12">
+        <v>327513.03236554743</v>
+      </c>
+      <c r="I7" s="12">
+        <v>367259.93340721406</v>
+      </c>
+      <c r="J7" s="12">
+        <v>407006.83444888087</v>
+      </c>
+      <c r="K7" s="12">
+        <v>446753.73549054749</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A8" s="10"/>
+      <c r="B8" s="170"/>
+      <c r="C8" s="122">
+        <f t="shared" si="1"/>
+        <v>0.13</v>
+      </c>
+      <c r="D8" s="12">
+        <v>226331.48334617523</v>
+      </c>
+      <c r="E8" s="12">
+        <v>269390.62614131428</v>
+      </c>
+      <c r="F8" s="12">
+        <v>312449.76893645315</v>
+      </c>
+      <c r="G8" s="12">
+        <v>355508.91173159186</v>
+      </c>
+      <c r="H8" s="12">
+        <v>398568.05452673091</v>
+      </c>
+      <c r="I8" s="12">
+        <v>441627.19732186978</v>
+      </c>
+      <c r="J8" s="12">
+        <v>484686.34011700866</v>
+      </c>
+      <c r="K8" s="12">
+        <v>527745.48291214765</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="A9" s="10"/>
+      <c r="B9" s="170"/>
+      <c r="C9" s="122">
+        <f t="shared" si="1"/>
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="D9" s="12">
+        <v>284137.53849346994</v>
+      </c>
+      <c r="E9" s="12">
+        <v>330508.92304208106</v>
+      </c>
+      <c r="F9" s="12">
+        <v>376880.30759069219</v>
+      </c>
+      <c r="G9" s="12">
+        <v>423251.69213930337</v>
+      </c>
+      <c r="H9" s="12">
+        <v>469623.07668791444</v>
+      </c>
+      <c r="I9" s="12">
+        <v>515994.46123652568</v>
+      </c>
+      <c r="J9" s="12">
+        <v>562365.8457851368</v>
+      </c>
+      <c r="K9" s="12">
+        <v>608737.23033374781</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B10" s="170"/>
+      <c r="C10" s="122">
+        <f t="shared" si="1"/>
+        <v>0.15000000000000002</v>
+      </c>
+      <c r="D10" s="12">
+        <v>341943.59364076459</v>
+      </c>
+      <c r="E10" s="12">
+        <v>391627.21994284791</v>
+      </c>
+      <c r="F10" s="12">
+        <v>441310.84624493145</v>
+      </c>
+      <c r="G10" s="12">
+        <v>490994.47254701483</v>
+      </c>
+      <c r="H10" s="12">
+        <v>540678.09884909808</v>
+      </c>
+      <c r="I10" s="12">
+        <v>590361.72515118145</v>
+      </c>
+      <c r="J10" s="12">
+        <v>640045.35145326494</v>
+      </c>
+      <c r="K10" s="12">
+        <v>689728.9777553482</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B11" s="170"/>
+      <c r="C11" s="122">
+        <f t="shared" si="1"/>
+        <v>0.16000000000000003</v>
+      </c>
+      <c r="D11" s="12">
+        <v>399749.64878805896</v>
+      </c>
+      <c r="E11" s="12">
+        <v>452745.51684361458</v>
+      </c>
+      <c r="F11" s="12">
+        <v>505741.38489917025</v>
+      </c>
+      <c r="G11" s="12">
+        <v>558737.25295472587</v>
+      </c>
+      <c r="H11" s="12">
+        <v>611733.12101028138</v>
+      </c>
+      <c r="I11" s="12">
+        <v>664728.989065837</v>
+      </c>
+      <c r="J11" s="12">
+        <v>717724.85712139274</v>
+      </c>
+      <c r="K11" s="12">
+        <v>770720.72517694836</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B12" s="170"/>
+      <c r="C12" s="122">
+        <f t="shared" si="1"/>
+        <v>0.17000000000000004</v>
+      </c>
+      <c r="D12" s="12">
+        <v>457555.70393535355</v>
+      </c>
+      <c r="E12" s="12">
+        <v>513863.81374438142</v>
+      </c>
+      <c r="F12" s="12">
+        <v>570171.92355340917</v>
+      </c>
+      <c r="G12" s="12">
+        <v>626480.03336243704</v>
+      </c>
+      <c r="H12" s="12">
+        <v>682788.14317146502</v>
+      </c>
+      <c r="I12" s="12">
+        <v>739096.25298049278</v>
+      </c>
+      <c r="J12" s="12">
+        <v>795404.36278952064</v>
+      </c>
+      <c r="K12" s="12">
+        <v>851712.47259854851</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B13" s="170"/>
+      <c r="C13" s="122">
+        <f t="shared" si="1"/>
+        <v>0.18000000000000005</v>
+      </c>
+      <c r="D13" s="12">
+        <v>515361.7590826482</v>
+      </c>
+      <c r="E13" s="12">
+        <v>574982.1106451482</v>
+      </c>
+      <c r="F13" s="12">
+        <v>634602.4622076482</v>
+      </c>
+      <c r="G13" s="12">
+        <v>694222.81377014844</v>
+      </c>
+      <c r="H13" s="12">
+        <v>753843.16533264855</v>
+      </c>
+      <c r="I13" s="12">
+        <v>813463.51689514844</v>
+      </c>
+      <c r="J13" s="12">
+        <v>873083.86845764844</v>
+      </c>
+      <c r="K13" s="12">
+        <v>932704.22002014832</v>
+      </c>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B14" s="170"/>
+      <c r="C14" s="122">
+        <f t="shared" si="1"/>
+        <v>0.19000000000000006</v>
+      </c>
+      <c r="D14" s="12">
+        <v>573167.81422994286</v>
+      </c>
+      <c r="E14" s="12">
+        <v>636100.40754591511</v>
+      </c>
+      <c r="F14" s="12">
+        <v>699033.00086188747</v>
+      </c>
+      <c r="G14" s="12">
+        <v>761965.59417785995</v>
+      </c>
+      <c r="H14" s="12">
+        <v>824898.18749383208</v>
+      </c>
+      <c r="I14" s="12">
+        <v>887830.78080980422</v>
+      </c>
+      <c r="J14" s="12">
+        <v>950763.3741257767</v>
+      </c>
+      <c r="K14" s="12">
+        <v>1013695.9674417488</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="B15" s="170"/>
+      <c r="C15" s="122">
+        <f t="shared" si="1"/>
+        <v>0.20000000000000007</v>
+      </c>
+      <c r="D15" s="12">
+        <v>630973.86937723751</v>
+      </c>
+      <c r="E15" s="12">
+        <v>697218.70444668189</v>
+      </c>
+      <c r="F15" s="12">
+        <v>763463.53951612674</v>
+      </c>
+      <c r="G15" s="12">
+        <v>829708.374585571</v>
+      </c>
+      <c r="H15" s="12">
+        <v>895953.20965501538</v>
+      </c>
+      <c r="I15" s="12">
+        <v>962198.04472446011</v>
+      </c>
+      <c r="J15" s="12">
+        <v>1028442.8797939043</v>
+      </c>
+      <c r="K15" s="12">
+        <v>1094687.7148633488</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>198</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B5:B15"/>
+    <mergeCell ref="D3:K3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9DFE4FD-5372-4920-8D3A-2456E7E15F04}">
   <dimension ref="B1:Z32"/>
@@ -7287,7 +8811,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92BEC192-FD1E-4512-A97A-EBF4BB0693FB}">
-  <dimension ref="A1:P62"/>
+  <dimension ref="A1:R62"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.6640625" style="85" customWidth="1"/>
@@ -7299,15 +8823,15 @@
     <col min="8" max="8" width="12.5" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.33203125" customWidth="1"/>
     <col min="10" max="10" width="18.5" customWidth="1"/>
-    <col min="11" max="11" width="36" customWidth="1"/>
-    <col min="12" max="12" width="23.33203125" customWidth="1"/>
-    <col min="13" max="13" width="15" customWidth="1"/>
-    <col min="14" max="14" width="15.5" customWidth="1"/>
-    <col min="15" max="15" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="19.6640625" customWidth="1"/>
+    <col min="11" max="13" width="36" customWidth="1"/>
+    <col min="14" max="14" width="23.33203125" customWidth="1"/>
+    <col min="15" max="15" width="15" customWidth="1"/>
+    <col min="16" max="16" width="15.5" customWidth="1"/>
+    <col min="17" max="17" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="19.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="113" t="s">
         <v>181</v>
       </c>
@@ -7342,10 +8866,16 @@
         <v>209</v>
       </c>
       <c r="L1" s="128" t="s">
+        <v>215</v>
+      </c>
+      <c r="M1" s="128" t="s">
+        <v>216</v>
+      </c>
+      <c r="N1" s="128" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="16" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" ht="16" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A2" s="114">
         <f>(1+'Project Details'!$F$5)^(B2/12)</f>
         <v>1</v>
@@ -7385,12 +8915,20 @@
         <f>SUM(C2:J2)</f>
         <v>77361.53</v>
       </c>
-      <c r="L2" s="64">
+      <c r="L2" s="112">
+        <f>SUM(C2:H2)/((1+'Project Details'!$F$6)^(B2/12))</f>
+        <v>-78158.47</v>
+      </c>
+      <c r="M2" s="112">
+        <f>SUM(I2:J2)/((1+'Project Details'!$F$6)^(B2/12))</f>
+        <v>155520</v>
+      </c>
+      <c r="N2" s="64">
         <f>K2</f>
         <v>77361.53</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" s="115">
         <f>(1+'Project Details'!$F$5)^(B3/12)</f>
         <v>1.0028708987190766</v>
@@ -7423,8 +8961,8 @@
         <v>-3662.9765907822116</v>
       </c>
       <c r="I3" s="33">
-        <f>IF(MOD(B3,12)=0,Revenue!$E$8*A3,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J3" s="119">
         <f>IF(MOD(B3,12)=0,Revenue!$E$4*A3,0)</f>
@@ -7432,14 +8970,22 @@
       </c>
       <c r="K3" s="112">
         <f>SUM(C3:J3)</f>
-        <v>-16038.425158616881</v>
-      </c>
-      <c r="L3" s="12">
+        <v>-10845.548446288114</v>
+      </c>
+      <c r="L3" s="112">
+        <f>SUM(C3:H3)/((1+'Project Details'!$F$6)^(B3/12))</f>
+        <v>-15935.893142309465</v>
+      </c>
+      <c r="M3" s="112">
+        <f>SUM(I3:J3)/((1+'Project Details'!$F$6)^(B3/12))</f>
+        <v>5159.6791811194862</v>
+      </c>
+      <c r="N3" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K3)</f>
-        <v>61425.636857690537</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+        <v>66585.316038810022</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4" s="115">
         <f>(1+'Project Details'!$F$5)^(B4/12)</f>
         <v>1.0057500394976084</v>
@@ -7472,8 +9018,8 @@
         <v>-3673.4926255846958</v>
       </c>
       <c r="I4" s="33">
-        <f>IF(MOD(B4,12)=0,Revenue!$E$8*A4,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J4" s="119">
         <f>IF(MOD(B4,12)=0,Revenue!$E$4*A4,0)</f>
@@ -7481,18 +9027,26 @@
       </c>
       <c r="K4" s="112">
         <f>SUM(C4:J4)</f>
-        <v>-16065.301243382688</v>
-      </c>
-      <c r="L4" s="12">
+        <v>-10872.424531053921</v>
+      </c>
+      <c r="L4" s="112">
+        <f>SUM(C4:H4)/((1+'Project Details'!$F$6)^(B4/12))</f>
+        <v>-15860.550153755923</v>
+      </c>
+      <c r="M4" s="112">
+        <f>SUM(I4:J4)/((1+'Project Details'!$F$6)^(B4/12))</f>
+        <v>5126.6938783414671</v>
+      </c>
+      <c r="N4" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K4)</f>
-        <v>45565.086703934605</v>
-      </c>
-      <c r="O4" s="129" t="s">
+        <v>55851.459763395564</v>
+      </c>
+      <c r="Q4" s="129" t="s">
         <v>184</v>
       </c>
-      <c r="P4" s="129"/>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="R4" s="129"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" s="115">
         <f>(1+'Project Details'!$F$5)^(B5/12)</f>
         <v>1.0086374459977134</v>
@@ -7525,30 +9079,38 @@
         <v>-3684.0388508580249</v>
       </c>
       <c r="I5" s="33">
-        <f>IF(MOD(B5,12)=0,Revenue!$E$8*A5,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J5" s="119">
         <f>IF(MOD(B5,12)=0,Revenue!$E$4*A5,0)</f>
         <v>0</v>
       </c>
       <c r="K5" s="112">
-        <f t="shared" ref="K5:K62" si="0">SUM(C5:J5)</f>
-        <v>-16092.254486665828</v>
-      </c>
-      <c r="L5" s="12">
+        <f>SUM(C5:J5)</f>
+        <v>-10899.377774337061</v>
+      </c>
+      <c r="L5" s="112">
+        <f>SUM(C5:H5)/((1+'Project Details'!$F$6)^(B5/12))</f>
+        <v>-15785.594887116262</v>
+      </c>
+      <c r="M5" s="112">
+        <f>SUM(I5:J5)/((1+'Project Details'!$F$6)^(B5/12))</f>
+        <v>5093.9194472399931</v>
+      </c>
+      <c r="N5" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K5)</f>
-        <v>29779.49181681835</v>
-      </c>
-      <c r="O5" s="1" t="s">
+        <v>45159.7843235193</v>
+      </c>
+      <c r="Q5" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="P5" s="12">
+      <c r="R5" s="12">
         <f>K2+NPV(('Project Details'!F6+1)^(1/12)-1,Cashflow!K3:K62)</f>
-        <v>185448.79524921341</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+        <v>168525.42819888081</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6" s="115">
         <f>(1+'Project Details'!$F$5)^(B6/12)</f>
         <v>1.0115331419494409</v>
@@ -7581,30 +9143,38 @@
         <v>-3694.6153532759813</v>
       </c>
       <c r="I6" s="33">
-        <f>IF(MOD(B6,12)=0,Revenue!$E$8*A6,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J6" s="119">
         <f>IF(MOD(B6,12)=0,Revenue!$E$4*A6,0)</f>
         <v>0</v>
       </c>
       <c r="K6" s="112">
-        <f t="shared" si="0"/>
-        <v>-16119.285109980579</v>
-      </c>
-      <c r="L6" s="12">
+        <f>SUM(C6:J6)</f>
+        <v>-10926.408397651812</v>
+      </c>
+      <c r="L6" s="112">
+        <f>SUM(C6:H6)/((1+'Project Details'!$F$6)^(B6/12))</f>
+        <v>-15711.025196297915</v>
+      </c>
+      <c r="M6" s="112">
+        <f>SUM(I6:J6)/((1+'Project Details'!$F$6)^(B6/12))</f>
+        <v>5061.3545397339421</v>
+      </c>
+      <c r="N6" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K6)</f>
-        <v>14068.466620520434</v>
-      </c>
-      <c r="O6" s="1" t="s">
+        <v>34510.113666955323</v>
+      </c>
+      <c r="Q6" s="1" t="s">
         <v>183</v>
       </c>
-      <c r="P6" s="13">
-        <f>-PMT('Project Details'!F6,'Project Details'!F4,Cashflow!P5)</f>
-        <v>46446.8477618092</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="R6" s="13">
+        <f>-PMT('Project Details'!F6,'Project Details'!F4,Cashflow!R5)</f>
+        <v>42208.281251049673</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" s="115">
         <f>(1+'Project Details'!$F$5)^(B7/12)</f>
         <v>1.0144371511509671</v>
@@ -7637,23 +9207,31 @@
         <v>-3705.2222197611823</v>
       </c>
       <c r="I7" s="33">
-        <f>IF(MOD(B7,12)=0,Revenue!$E$8*A7,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J7" s="119">
         <f>IF(MOD(B7,12)=0,Revenue!$E$4*A7,0)</f>
         <v>0</v>
       </c>
       <c r="K7" s="112">
-        <f t="shared" si="0"/>
-        <v>-16146.393335477182</v>
-      </c>
-      <c r="L7" s="12">
+        <f>SUM(C7:J7)</f>
+        <v>-10953.516623148415</v>
+      </c>
+      <c r="L7" s="112">
+        <f>SUM(C7:H7)/((1+'Project Details'!$F$6)^(B7/12))</f>
+        <v>-15636.838947750659</v>
+      </c>
+      <c r="M7" s="112">
+        <f>SUM(I7:J7)/((1+'Project Details'!$F$6)^(B7/12))</f>
+        <v>5028.9978163603382</v>
+      </c>
+      <c r="N7" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K7)</f>
-        <v>-1568.3723272302159</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+        <v>23902.272535565004</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8" s="115">
         <f>(1+'Project Details'!$F$5)^(B8/12)</f>
         <v>1.0173494974687902</v>
@@ -7686,23 +9264,31 @@
         <v>-3715.8595374857891</v>
       </c>
       <c r="I8" s="33">
-        <f>IF(MOD(B8,12)=0,Revenue!$E$8*A8,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J8" s="119">
         <f>IF(MOD(B8,12)=0,Revenue!$E$4*A8,0)</f>
         <v>0</v>
       </c>
       <c r="K8" s="112">
-        <f t="shared" si="0"/>
-        <v>-16173.57938594364</v>
-      </c>
-      <c r="L8" s="12">
+        <f>SUM(C8:J8)</f>
+        <v>-10980.702673614873</v>
+      </c>
+      <c r="L8" s="112">
+        <f>SUM(C8:H8)/((1+'Project Details'!$F$6)^(B8/12))</f>
+        <v>-15563.034020390569</v>
+      </c>
+      <c r="M8" s="112">
+        <f>SUM(I8:J8)/((1+'Project Details'!$F$6)^(B8/12))</f>
+        <v>4996.8479462192536</v>
+      </c>
+      <c r="N8" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K8)</f>
-        <v>-17131.406347620781</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+        <v>13336.086461393679</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" s="115">
         <f>(1+'Project Details'!$F$5)^(B9/12)</f>
         <v>1.0202702048379266</v>
@@ -7735,23 +9321,31 @@
         <v>-3726.5273938722257</v>
       </c>
       <c r="I9" s="33">
-        <f>IF(MOD(B9,12)=0,Revenue!$E$8*A9,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J9" s="119">
         <f>IF(MOD(B9,12)=0,Revenue!$E$4*A9,0)</f>
         <v>0</v>
       </c>
       <c r="K9" s="112">
-        <f t="shared" si="0"/>
-        <v>-16200.843484807561</v>
-      </c>
-      <c r="L9" s="12">
+        <f>SUM(C9:J9)</f>
+        <v>-11007.966772478794</v>
+      </c>
+      <c r="L9" s="112">
+        <f>SUM(C9:H9)/((1+'Project Details'!$F$6)^(B9/12))</f>
+        <v>-15489.608305524496</v>
+      </c>
+      <c r="M9" s="112">
+        <f>SUM(I9:J9)/((1+'Project Details'!$F$6)^(B9/12))</f>
+        <v>4964.9036069190715</v>
+      </c>
+      <c r="N9" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K9)</f>
-        <v>-32621.014653145292</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+        <v>2811.3817627882527</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10" s="115">
         <f>(1+'Project Details'!$F$5)^(B10/12)</f>
         <v>1.0231992972621078</v>
@@ -7784,23 +9378,31 @@
         <v>-3737.2258765938968</v>
       </c>
       <c r="I10" s="33">
-        <f>IF(MOD(B10,12)=0,Revenue!$E$8*A10,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J10" s="119">
         <f>IF(MOD(B10,12)=0,Revenue!$E$4*A10,0)</f>
         <v>0</v>
       </c>
       <c r="K10" s="112">
-        <f t="shared" si="0"/>
-        <v>-16228.185856137981</v>
-      </c>
-      <c r="L10" s="12">
+        <f>SUM(C10:J10)</f>
+        <v>-11035.309143809214</v>
+      </c>
+      <c r="L10" s="112">
+        <f>SUM(C10:H10)/((1+'Project Details'!$F$6)^(B10/12))</f>
+        <v>-15416.559706774959</v>
+      </c>
+      <c r="M10" s="112">
+        <f>SUM(I10:J10)/((1+'Project Details'!$F$6)^(B10/12))</f>
+        <v>4933.1634845220869</v>
+      </c>
+      <c r="N10" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K10)</f>
-        <v>-48037.574359920254</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+        <v>-7672.0144594646117</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11" s="115">
         <f>(1+'Project Details'!$F$5)^(B11/12)</f>
         <v>1.0261367988139778</v>
@@ -7833,23 +9435,31 @@
         <v>-3747.9550735759108</v>
       </c>
       <c r="I11" s="33">
-        <f>IF(MOD(B11,12)=0,Revenue!$E$8*A11,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J11" s="119">
         <f>IF(MOD(B11,12)=0,Revenue!$E$4*A11,0)</f>
         <v>0</v>
       </c>
       <c r="K11" s="112">
-        <f t="shared" si="0"/>
-        <v>-16255.606724647238</v>
-      </c>
-      <c r="L11" s="12">
+        <f>SUM(C11:J11)</f>
+        <v>-11062.73001231847</v>
+      </c>
+      <c r="L11" s="112">
+        <f>SUM(C11:H11)/((1+'Project Details'!$F$6)^(B11/12))</f>
+        <v>-15343.886140005596</v>
+      </c>
+      <c r="M11" s="112">
+        <f>SUM(I11:J11)/((1+'Project Details'!$F$6)^(B11/12))</f>
+        <v>4901.6262734904658</v>
+      </c>
+      <c r="N11" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K11)</f>
-        <v>-63381.460499925859</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+        <v>-18114.274325979757</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12" s="115">
         <f>(1+'Project Details'!$F$5)^(B12/12)</f>
         <v>1.0290827336352901</v>
@@ -7882,23 +9492,31 @@
         <v>-3758.7150729957962</v>
       </c>
       <c r="I12" s="33">
-        <f>IF(MOD(B12,12)=0,Revenue!$E$8*A12,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J12" s="119">
         <f>IF(MOD(B12,12)=0,Revenue!$E$4*A12,0)</f>
         <v>0</v>
       </c>
       <c r="K12" s="112">
-        <f t="shared" si="0"/>
-        <v>-16283.106315692767</v>
-      </c>
-      <c r="L12" s="12">
+        <f>SUM(C12:J12)</f>
+        <v>-11090.229603364</v>
+      </c>
+      <c r="L12" s="112">
+        <f>SUM(C12:H12)/((1+'Project Details'!$F$6)^(B12/12))</f>
+        <v>-15271.585533246945</v>
+      </c>
+      <c r="M12" s="112">
+        <f>SUM(I12:J12)/((1+'Project Details'!$F$6)^(B12/12))</f>
+        <v>4870.2906766325432</v>
+      </c>
+      <c r="N12" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K12)</f>
-        <v>-78653.046033172839</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+        <v>-28515.569182594161</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A13" s="115">
         <f>(1+'Project Details'!$F$5)^(B13/12)</f>
         <v>1.0320371259371075</v>
@@ -7931,23 +9549,31 @@
         <v>-3769.5059632842335</v>
       </c>
       <c r="I13" s="33">
-        <f>IF(MOD(B13,12)=0,Revenue!$E$8*A13,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J13" s="119">
         <f>IF(MOD(B13,12)=0,Revenue!$E$4*A13,0)</f>
         <v>0</v>
       </c>
       <c r="K13" s="112">
-        <f t="shared" si="0"/>
-        <v>-16310.684855279007</v>
-      </c>
-      <c r="L13" s="12">
+        <f>SUM(C13:J13)</f>
+        <v>-11117.80814295024</v>
+      </c>
+      <c r="L13" s="112">
+        <f>SUM(C13:H13)/((1+'Project Details'!$F$6)^(B13/12))</f>
+        <v>-15199.65582662282</v>
+      </c>
+      <c r="M13" s="112">
+        <f>SUM(I13:J13)/((1+'Project Details'!$F$6)^(B13/12))</f>
+        <v>4839.1554050494678</v>
+      </c>
+      <c r="N13" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K13)</f>
-        <v>-93852.701859795663</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+        <v>-38876.069604167511</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A14" s="115">
         <f>(1+'Project Details'!$F$5)^(B14/12)</f>
         <v>1.0349999999999999</v>
@@ -7980,23 +9606,31 @@
         <v>-3780.3278331257784</v>
       </c>
       <c r="I14" s="33">
-        <f>IF(MOD(B14,12)=0,Revenue!$E$8*A14,0)</f>
-        <v>64495.52876712328</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J14" s="119">
         <f>IF(MOD(B14,12)=0,Revenue!$E$4*A14,0)</f>
         <v>160963.19999999998</v>
       </c>
       <c r="K14" s="112">
-        <f t="shared" si="0"/>
-        <v>206532.88619706404</v>
-      </c>
-      <c r="L14" s="12">
+        <f>SUM(C14:J14)</f>
+        <v>147230.23414226953</v>
+      </c>
+      <c r="L14" s="112">
+        <f>SUM(C14:H14)/((1+'Project Details'!$F$6)^(B14/12))</f>
+        <v>-17523.928305610389</v>
+      </c>
+      <c r="M14" s="112">
+        <f>SUM(I14:J14)/((1+'Project Details'!$F$6)^(B14/12))</f>
+        <v>153848.21917808216</v>
+      </c>
+      <c r="N14" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K14)</f>
-        <v>97381.452026374813</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+        <v>97448.221268304318</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A15" s="115">
         <f>(1+'Project Details'!$F$5)^(B15/12)</f>
         <v>1.0379713801742443</v>
@@ -8029,23 +9663,31 @@
         <v>-3791.1807714595889</v>
       </c>
       <c r="I15" s="33">
-        <f>IF(MOD(B15,12)=0,Revenue!$E$8*A15,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J15" s="119">
         <f>IF(MOD(B15,12)=0,Revenue!$E$4*A15,0)</f>
         <v>0</v>
       </c>
       <c r="K15" s="112">
-        <f t="shared" si="0"/>
-        <v>-16366.079687337366</v>
-      </c>
-      <c r="L15" s="12">
+        <f>SUM(C15:J15)</f>
+        <v>-11173.202975008599</v>
+      </c>
+      <c r="L15" s="112">
+        <f>SUM(C15:H15)/((1+'Project Details'!$F$6)^(B15/12))</f>
+        <v>-15056.900934300709</v>
+      </c>
+      <c r="M15" s="112">
+        <f>SUM(I15:J15)/((1+'Project Details'!$F$6)^(B15/12))</f>
+        <v>4777.4807232587837</v>
+      </c>
+      <c r="N15" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K15)</f>
-        <v>82324.551092074093</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+        <v>87168.80105726239</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A16" s="115">
         <f>(1+'Project Details'!$F$5)^(B16/12)</f>
         <v>1.0409512908800247</v>
@@ -8078,23 +9720,31 @@
         <v>-3802.06486748016</v>
       </c>
       <c r="I16" s="33">
-        <f>IF(MOD(B16,12)=0,Revenue!$E$8*A16,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J16" s="119">
         <f>IF(MOD(B16,12)=0,Revenue!$E$4*A16,0)</f>
         <v>0</v>
       </c>
       <c r="K16" s="112">
-        <f t="shared" si="0"/>
-        <v>-16393.896435069979</v>
-      </c>
-      <c r="L16" s="12">
+        <f>SUM(C16:J16)</f>
+        <v>-11201.019722741212</v>
+      </c>
+      <c r="L16" s="112">
+        <f>SUM(C16:H16)/((1+'Project Details'!$F$6)^(B16/12))</f>
+        <v>-14986.071688659775</v>
+      </c>
+      <c r="M16" s="112">
+        <f>SUM(I16:J16)/((1+'Project Details'!$F$6)^(B16/12))</f>
+        <v>4746.9387762420984</v>
+      </c>
+      <c r="N16" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K16)</f>
-        <v>67338.479403414312</v>
-      </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+        <v>76929.668144844705</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A17" s="115">
         <f>(1+'Project Details'!$F$5)^(B17/12)</f>
         <v>1.0439397566076332</v>
@@ -8127,23 +9777,31 @@
         <v>-3812.9802106380548</v>
       </c>
       <c r="I17" s="33">
-        <f>IF(MOD(B17,12)=0,Revenue!$E$8*A17,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J17" s="119">
         <f>IF(MOD(B17,12)=0,Revenue!$E$4*A17,0)</f>
         <v>0</v>
       </c>
       <c r="K17" s="112">
-        <f t="shared" si="0"/>
-        <v>-16421.793041868026</v>
-      </c>
-      <c r="L17" s="12">
+        <f>SUM(C17:J17)</f>
+        <v>-11228.916329539259</v>
+      </c>
+      <c r="L17" s="112">
+        <f>SUM(C17:H17)/((1+'Project Details'!$F$6)^(B17/12))</f>
+        <v>-14915.605223123284</v>
+      </c>
+      <c r="M17" s="112">
+        <f>SUM(I17:J17)/((1+'Project Details'!$F$6)^(B17/12))</f>
+        <v>4716.5920807777702</v>
+      </c>
+      <c r="N17" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K17)</f>
-        <v>52422.874180291015</v>
-      </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+        <v>66730.655002499188</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A18" s="115">
         <f>(1+'Project Details'!$F$5)^(B18/12)</f>
         <v>1.0469368019176712</v>
@@ -8176,23 +9834,31 @@
         <v>-3823.9268906406401</v>
       </c>
       <c r="I18" s="33">
-        <f>IF(MOD(B18,12)=0,Revenue!$E$8*A18,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J18" s="119">
         <f>IF(MOD(B18,12)=0,Revenue!$E$4*A18,0)</f>
         <v>0</v>
       </c>
       <c r="K18" s="112">
-        <f t="shared" si="0"/>
-        <v>-16449.769736998795</v>
-      </c>
-      <c r="L18" s="12">
+        <f>SUM(C18:J18)</f>
+        <v>-11256.893024670027</v>
+      </c>
+      <c r="L18" s="112">
+        <f>SUM(C18:H18)/((1+'Project Details'!$F$6)^(B18/12))</f>
+        <v>-14845.499537191872</v>
+      </c>
+      <c r="M18" s="112">
+        <f>SUM(I18:J18)/((1+'Project Details'!$F$6)^(B18/12))</f>
+        <v>4686.4393886425387</v>
+      </c>
+      <c r="N18" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K18)</f>
-        <v>37577.37464309913</v>
-      </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+        <v>56571.594853949849</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A19" s="115">
         <f>(1+'Project Details'!$F$5)^(B19/12)</f>
         <v>1.049942451441251</v>
@@ -8225,23 +9891,31 @@
         <v>-3834.9049974528234</v>
       </c>
       <c r="I19" s="33">
-        <f>IF(MOD(B19,12)=0,Revenue!$E$8*A19,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J19" s="119">
         <f>IF(MOD(B19,12)=0,Revenue!$E$4*A19,0)</f>
         <v>0</v>
       </c>
       <c r="K19" s="112">
-        <f t="shared" si="0"/>
-        <v>-16477.82675038778</v>
-      </c>
-      <c r="L19" s="12">
+        <f>SUM(C19:J19)</f>
+        <v>-11284.950038059013</v>
+      </c>
+      <c r="L19" s="112">
+        <f>SUM(C19:H19)/((1+'Project Details'!$F$6)^(B19/12))</f>
+        <v>-14775.752642026795</v>
+      </c>
+      <c r="M19" s="112">
+        <f>SUM(I19:J19)/((1+'Project Details'!$F$6)^(B19/12))</f>
+        <v>4656.4794595929052</v>
+      </c>
+      <c r="N19" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K19)</f>
-        <v>22801.622001072326</v>
-      </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+        <v>46452.321671515951</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A20" s="115">
         <f>(1+'Project Details'!$F$5)^(B20/12)</f>
         <v>1.0529567298801978</v>
@@ -8274,23 +9948,31 @@
         <v>-3845.9146212977912</v>
       </c>
       <c r="I20" s="33">
-        <f>IF(MOD(B20,12)=0,Revenue!$E$8*A20,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J20" s="119">
         <f>IF(MOD(B20,12)=0,Revenue!$E$4*A20,0)</f>
         <v>0</v>
       </c>
       <c r="K20" s="112">
-        <f t="shared" si="0"/>
-        <v>-16505.964312620563</v>
-      </c>
-      <c r="L20" s="12">
+        <f>SUM(C20:J20)</f>
+        <v>-11313.087600291796</v>
+      </c>
+      <c r="L20" s="112">
+        <f>SUM(C20:H20)/((1+'Project Details'!$F$6)^(B20/12))</f>
+        <v>-14706.362560379379</v>
+      </c>
+      <c r="M20" s="112">
+        <f>SUM(I20:J20)/((1+'Project Details'!$F$6)^(B20/12))</f>
+        <v>4626.711061314124</v>
+      </c>
+      <c r="N20" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K20)</f>
-        <v>8095.2594406929275</v>
-      </c>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+        <v>36372.670172450693</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A21" s="115">
         <f>(1+'Project Details'!$F$5)^(B21/12)</f>
         <v>1.0559796620072539</v>
@@ -8323,23 +10005,31 @@
         <v>-3856.955852657753</v>
       </c>
       <c r="I21" s="33">
-        <f>IF(MOD(B21,12)=0,Revenue!$E$8*A21,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J21" s="119">
         <f>IF(MOD(B21,12)=0,Revenue!$E$4*A21,0)</f>
         <v>0</v>
       </c>
       <c r="K21" s="112">
-        <f t="shared" si="0"/>
-        <v>-16534.182654944718</v>
-      </c>
-      <c r="L21" s="12">
+        <f>SUM(C21:J21)</f>
+        <v>-11341.305942615951</v>
+      </c>
+      <c r="L21" s="112">
+        <f>SUM(C21:H21)/((1+'Project Details'!$F$6)^(B21/12))</f>
+        <v>-14637.327326520901</v>
+      </c>
+      <c r="M21" s="112">
+        <f>SUM(I21:J21)/((1+'Project Details'!$F$6)^(B21/12))</f>
+        <v>4597.1329693695106</v>
+      </c>
+      <c r="N21" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K21)</f>
-        <v>-6542.0678858279716</v>
-      </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+        <v>26332.475815299302</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A22" s="115">
         <f>(1+'Project Details'!$F$5)^(B22/12)</f>
         <v>1.0590112726662815</v>
@@ -8372,23 +10062,31 @@
         <v>-3868.0287822746832</v>
       </c>
       <c r="I22" s="33">
-        <f>IF(MOD(B22,12)=0,Revenue!$E$8*A22,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J22" s="119">
         <f>IF(MOD(B22,12)=0,Revenue!$E$4*A22,0)</f>
         <v>0</v>
       </c>
       <c r="K22" s="112">
-        <f t="shared" si="0"/>
-        <v>-16562.482009271705</v>
-      </c>
-      <c r="L22" s="12">
+        <f>SUM(C22:J22)</f>
+        <v>-11369.605296942938</v>
+      </c>
+      <c r="L22" s="112">
+        <f>SUM(C22:H22)/((1+'Project Details'!$F$6)^(B22/12))</f>
+        <v>-14568.644986172914</v>
+      </c>
+      <c r="M22" s="112">
+        <f>SUM(I22:J22)/((1+'Project Details'!$F$6)^(B22/12))</f>
+        <v>4567.7439671500806</v>
+      </c>
+      <c r="N22" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K22)</f>
-        <v>-21110.712872000906</v>
-      </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+        <v>16331.574796276458</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A23" s="115">
         <f>(1+'Project Details'!$F$5)^(B23/12)</f>
         <v>1.0620515867724669</v>
@@ -8421,23 +10119,31 @@
         <v>-3879.1335011510673</v>
       </c>
       <c r="I23" s="33">
-        <f>IF(MOD(B23,12)=0,Revenue!$E$8*A23,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J23" s="119">
         <f>IF(MOD(B23,12)=0,Revenue!$E$4*A23,0)</f>
         <v>0</v>
       </c>
       <c r="K23" s="112">
-        <f t="shared" si="0"/>
-        <v>-16590.862608178784</v>
-      </c>
-      <c r="L23" s="12">
+        <f>SUM(C23:J23)</f>
+        <v>-11397.985895850017</v>
+      </c>
+      <c r="L23" s="112">
+        <f>SUM(C23:H23)/((1+'Project Details'!$F$6)^(B23/12))</f>
+        <v>-14500.313596438005</v>
+      </c>
+      <c r="M23" s="112">
+        <f>SUM(I23:J23)/((1+'Project Details'!$F$6)^(B23/12))</f>
+        <v>4538.5428458245051</v>
+      </c>
+      <c r="N23" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K23)</f>
-        <v>-35611.026468438926</v>
-      </c>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+        <v>6369.8040456629533</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A24" s="115">
         <f>(1+'Project Details'!$F$5)^(B24/12)</f>
         <v>1.0651006293125251</v>
@@ -8470,23 +10176,31 @@
         <v>-3890.2701005506487</v>
       </c>
       <c r="I24" s="33">
-        <f>IF(MOD(B24,12)=0,Revenue!$E$8*A24,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J24" s="119">
         <f>IF(MOD(B24,12)=0,Revenue!$E$4*A24,0)</f>
         <v>0</v>
       </c>
       <c r="K24" s="112">
-        <f t="shared" si="0"/>
-        <v>-16619.324684910909</v>
-      </c>
-      <c r="L24" s="12">
+        <f>SUM(C24:J24)</f>
+        <v>-11426.447972582142</v>
+      </c>
+      <c r="L24" s="112">
+        <f>SUM(C24:H24)/((1+'Project Details'!$F$6)^(B24/12))</f>
+        <v>-14432.331225730955</v>
+      </c>
+      <c r="M24" s="112">
+        <f>SUM(I24:J24)/((1+'Project Details'!$F$6)^(B24/12))</f>
+        <v>4509.5284042893909</v>
+      </c>
+      <c r="N24" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K24)</f>
-        <v>-50043.357694169885</v>
-      </c>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+        <v>-3552.9987757786148</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A25" s="115">
         <f>(1+'Project Details'!$F$5)^(B25/12)</f>
         <v>1.0681584253449063</v>
@@ -8519,23 +10233,31 @@
         <v>-3901.4386719991821</v>
       </c>
       <c r="I25" s="33">
-        <f>IF(MOD(B25,12)=0,Revenue!$E$8*A25,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J25" s="119">
         <f>IF(MOD(B25,12)=0,Revenue!$E$4*A25,0)</f>
         <v>0</v>
       </c>
       <c r="K25" s="112">
-        <f t="shared" si="0"/>
-        <v>-16647.868473382667</v>
-      </c>
-      <c r="L25" s="12">
+        <f>SUM(C25:J25)</f>
+        <v>-11454.9917610539</v>
+      </c>
+      <c r="L25" s="112">
+        <f>SUM(C25:H25)/((1+'Project Details'!$F$6)^(B25/12))</f>
+        <v>-14364.695953710378</v>
+      </c>
+      <c r="M25" s="112">
+        <f>SUM(I25:J25)/((1+'Project Details'!$F$6)^(B25/12))</f>
+        <v>4480.6994491198775</v>
+      </c>
+      <c r="N25" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K25)</f>
-        <v>-64408.053647880268</v>
-      </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+        <v>-13436.995280369127</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A26" s="115">
         <f>(1+'Project Details'!$F$5)^(B26/12)</f>
         <v>1.0712249999999999</v>
@@ -8568,23 +10290,31 @@
         <v>-3912.6393072851806</v>
       </c>
       <c r="I26" s="33">
-        <f>IF(MOD(B26,12)=0,Revenue!$E$8*A26,0)</f>
-        <v>66752.872273972593</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J26" s="119">
         <f>IF(MOD(B26,12)=0,Revenue!$E$4*A26,0)</f>
         <v>166596.91199999998</v>
       </c>
       <c r="K26" s="112">
-        <f t="shared" si="0"/>
-        <v>213995.22756579239</v>
-      </c>
-      <c r="L26" s="12">
+        <f>SUM(C26:J26)</f>
+        <v>152435.23200414857</v>
+      </c>
+      <c r="L26" s="112">
+        <f>SUM(C26:H26)/((1+'Project Details'!$F$6)^(B26/12))</f>
+        <v>-16593.412815655163</v>
+      </c>
+      <c r="M26" s="112">
+        <f>SUM(I26:J26)/((1+'Project Details'!$F$6)^(B26/12))</f>
+        <v>147282.05479452052</v>
+      </c>
+      <c r="N26" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K26)</f>
-        <v>119058.36230358796</v>
-      </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+        <v>117251.64669849635</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A27" s="115">
         <f>(1+'Project Details'!$F$5)^(B27/12)</f>
         <v>1.0743003784803427</v>
@@ -8617,23 +10347,31 @@
         <v>-3923.8720984606739</v>
       </c>
       <c r="I27" s="33">
-        <f>IF(MOD(B27,12)=0,Revenue!$E$8*A27,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J27" s="119">
         <f>IF(MOD(B27,12)=0,Revenue!$E$4*A27,0)</f>
         <v>0</v>
       </c>
       <c r="K27" s="112">
-        <f t="shared" si="0"/>
-        <v>-16705.202124563068</v>
-      </c>
-      <c r="L27" s="12">
+        <f>SUM(C27:J27)</f>
+        <v>-11512.325412234301</v>
+      </c>
+      <c r="L27" s="112">
+        <f>SUM(C27:H27)/((1+'Project Details'!$F$6)^(B27/12))</f>
+        <v>-14230.459080174724</v>
+      </c>
+      <c r="M27" s="112">
+        <f>SUM(I27:J27)/((1+'Project Details'!$F$6)^(B27/12))</f>
+        <v>4423.5932622766504</v>
+      </c>
+      <c r="N27" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K27)</f>
-        <v>104827.90322341322</v>
-      </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+        <v>107444.78088059826</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A28" s="115">
         <f>(1+'Project Details'!$F$5)^(B28/12)</f>
         <v>1.0773845860608253</v>
@@ -8666,23 +10404,31 @@
         <v>-3935.1371378419649</v>
       </c>
       <c r="I28" s="33">
-        <f>IF(MOD(B28,12)=0,Revenue!$E$8*A28,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J28" s="119">
         <f>IF(MOD(B28,12)=0,Revenue!$E$4*A28,0)</f>
         <v>0</v>
       </c>
       <c r="K28" s="112">
-        <f t="shared" si="0"/>
-        <v>-16733.99245846632</v>
-      </c>
-      <c r="L28" s="12">
+        <f>SUM(C28:J28)</f>
+        <v>-11541.115746137553</v>
+      </c>
+      <c r="L28" s="112">
+        <f>SUM(C28:H28)/((1+'Project Details'!$F$6)^(B28/12))</f>
+        <v>-14163.853693586307</v>
+      </c>
+      <c r="M28" s="112">
+        <f>SUM(I28:J28)/((1+'Project Details'!$F$6)^(B28/12))</f>
+        <v>4395.3136817056466</v>
+      </c>
+      <c r="N28" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K28)</f>
-        <v>90664.049529826894</v>
-      </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+        <v>97676.240868717607</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A29" s="115">
         <f>(1+'Project Details'!$F$5)^(B29/12)</f>
         <v>1.0804776480889005</v>
@@ -8715,23 +10461,31 @@
         <v>-3946.4345180103869</v>
       </c>
       <c r="I29" s="33">
-        <f>IF(MOD(B29,12)=0,Revenue!$E$8*A29,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J29" s="119">
         <f>IF(MOD(B29,12)=0,Revenue!$E$4*A29,0)</f>
         <v>0</v>
       </c>
       <c r="K29" s="112">
-        <f t="shared" si="0"/>
-        <v>-16762.865446502303</v>
-      </c>
-      <c r="L29" s="12">
+        <f>SUM(C29:J29)</f>
+        <v>-11569.988734173536</v>
+      </c>
+      <c r="L29" s="112">
+        <f>SUM(C29:H29)/((1+'Project Details'!$F$6)^(B29/12))</f>
+        <v>-14097.587835403829</v>
+      </c>
+      <c r="M29" s="112">
+        <f>SUM(I29:J29)/((1+'Project Details'!$F$6)^(B29/12))</f>
+        <v>4367.2148896090466</v>
+      </c>
+      <c r="N29" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K29)</f>
-        <v>76566.461694423051</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+        <v>87945.8679229228</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A30" s="115">
         <f>(1+'Project Details'!$F$5)^(B30/12)</f>
         <v>1.0835795899847898</v>
@@ -8764,23 +10518,31 @@
         <v>-3957.7643318130627</v>
       </c>
       <c r="I30" s="33">
-        <f>IF(MOD(B30,12)=0,Revenue!$E$8*A30,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J30" s="119">
         <f>IF(MOD(B30,12)=0,Revenue!$E$4*A30,0)</f>
         <v>0</v>
       </c>
       <c r="K30" s="112">
-        <f t="shared" si="0"/>
-        <v>-16791.821325962646</v>
-      </c>
-      <c r="L30" s="12">
+        <f>SUM(C30:J30)</f>
+        <v>-11598.944613633879</v>
+      </c>
+      <c r="L30" s="112">
+        <f>SUM(C30:H30)/((1+'Project Details'!$F$6)^(B30/12))</f>
+        <v>-14031.659640493786</v>
+      </c>
+      <c r="M30" s="112">
+        <f>SUM(I30:J30)/((1+'Project Details'!$F$6)^(B30/12))</f>
+        <v>4339.2957302245723</v>
+      </c>
+      <c r="N30" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K30)</f>
-        <v>62534.802053929248</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+        <v>78253.504012653575</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A31" s="115">
         <f>(1+'Project Details'!$F$5)^(B31/12)</f>
         <v>1.0866904372416946</v>
@@ -8813,23 +10575,31 @@
         <v>-3969.1266723636718</v>
       </c>
       <c r="I31" s="33">
-        <f>IF(MOD(B31,12)=0,Revenue!$E$8*A31,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J31" s="119">
         <f>IF(MOD(B31,12)=0,Revenue!$E$4*A31,0)</f>
         <v>0</v>
       </c>
       <c r="K31" s="112">
-        <f t="shared" si="0"/>
-        <v>-16820.860334820245</v>
-      </c>
-      <c r="L31" s="12">
+        <f>SUM(C31:J31)</f>
+        <v>-11627.983622491478</v>
+      </c>
+      <c r="L31" s="112">
+        <f>SUM(C31:H31)/((1+'Project Details'!$F$6)^(B31/12))</f>
+        <v>-13966.067254564949</v>
+      </c>
+      <c r="M31" s="112">
+        <f>SUM(I31:J31)/((1+'Project Details'!$F$6)^(B31/12))</f>
+        <v>4311.5550551786155</v>
+      </c>
+      <c r="N31" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K31)</f>
-        <v>48568.734799364283</v>
-      </c>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+        <v>68598.991813267232</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A32" s="115">
         <f>(1+'Project Details'!$F$5)^(B32/12)</f>
         <v>1.0898102154260045</v>
@@ -8862,23 +10632,31 @@
         <v>-3980.5216330432131</v>
       </c>
       <c r="I32" s="33">
-        <f>IF(MOD(B32,12)=0,Revenue!$E$8*A32,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J32" s="119">
         <f>IF(MOD(B32,12)=0,Revenue!$E$4*A32,0)</f>
         <v>0</v>
       </c>
       <c r="K32" s="112">
-        <f t="shared" si="0"/>
-        <v>-16849.982711731176</v>
-      </c>
-      <c r="L32" s="12">
+        <f>SUM(C32:J32)</f>
+        <v>-11657.105999402409</v>
+      </c>
+      <c r="L32" s="112">
+        <f>SUM(C32:H32)/((1+'Project Details'!$F$6)^(B32/12))</f>
+        <v>-13900.808834102842</v>
+      </c>
+      <c r="M32" s="112">
+        <f>SUM(I32:J32)/((1+'Project Details'!$F$6)^(B32/12))</f>
+        <v>4283.9917234390032</v>
+      </c>
+      <c r="N32" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K32)</f>
-        <v>34667.925965261427</v>
-      </c>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.2">
+        <v>58982.174702603392</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A33" s="115">
         <f>(1+'Project Details'!$F$5)^(B33/12)</f>
         <v>1.0929389501775078</v>
@@ -8911,23 +10689,31 @@
         <v>-3991.949307500774</v>
       </c>
       <c r="I33" s="33">
-        <f>IF(MOD(B33,12)=0,Revenue!$E$8*A33,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J33" s="119">
         <f>IF(MOD(B33,12)=0,Revenue!$E$4*A33,0)</f>
         <v>0</v>
       </c>
       <c r="K33" s="112">
-        <f t="shared" si="0"/>
-        <v>-16879.188696036676</v>
-      </c>
-      <c r="L33" s="12">
+        <f>SUM(C33:J33)</f>
+        <v>-11686.311983707908</v>
+      </c>
+      <c r="L33" s="112">
+        <f>SUM(C33:H33)/((1+'Project Details'!$F$6)^(B33/12))</f>
+        <v>-13835.882546304683</v>
+      </c>
+      <c r="M33" s="112">
+        <f>SUM(I33:J33)/((1+'Project Details'!$F$6)^(B33/12))</f>
+        <v>4256.6046012680654</v>
+      </c>
+      <c r="N33" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K33)</f>
-        <v>20832.043418956731</v>
-      </c>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.2">
+        <v>49402.896757566763</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A34" s="115">
         <f>(1+'Project Details'!$F$5)^(B34/12)</f>
         <v>1.0960766672096012</v>
@@ -8960,23 +10746,31 @@
         <v>-4003.4097896542962</v>
       </c>
       <c r="I34" s="33">
-        <f>IF(MOD(B34,12)=0,Revenue!$E$8*A34,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J34" s="119">
         <f>IF(MOD(B34,12)=0,Revenue!$E$4*A34,0)</f>
         <v>0</v>
       </c>
       <c r="K34" s="112">
-        <f t="shared" si="0"/>
-        <v>-16908.47852776511</v>
-      </c>
-      <c r="L34" s="12">
+        <f>SUM(C34:J34)</f>
+        <v>-11715.601815436343</v>
+      </c>
+      <c r="L34" s="112">
+        <f>SUM(C34:H34)/((1+'Project Details'!$F$6)^(B34/12))</f>
+        <v>-13771.286569014701</v>
+      </c>
+      <c r="M34" s="112">
+        <f>SUM(I34:J34)/((1+'Project Details'!$F$6)^(B34/12))</f>
+        <v>4229.392562176</v>
+      </c>
+      <c r="N34" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K34)</f>
-        <v>7060.7568499420158</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.2">
+        <v>39861.002750728054</v>
+      </c>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A35" s="115">
         <f>(1+'Project Details'!$F$5)^(B35/12)</f>
         <v>1.0992233923095032</v>
@@ -9009,23 +10803,31 @@
         <v>-4014.9031736913544</v>
       </c>
       <c r="I35" s="33">
-        <f>IF(MOD(B35,12)=0,Revenue!$E$8*A35,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J35" s="119">
         <f>IF(MOD(B35,12)=0,Revenue!$E$4*A35,0)</f>
         <v>0</v>
       </c>
       <c r="K35" s="112">
-        <f t="shared" si="0"/>
-        <v>-16937.852447633937</v>
-      </c>
-      <c r="L35" s="12">
+        <f>SUM(C35:J35)</f>
+        <v>-11744.97573530517</v>
+      </c>
+      <c r="L35" s="112">
+        <f>SUM(C35:H35)/((1+'Project Details'!$F$6)^(B35/12))</f>
+        <v>-13707.019090659856</v>
+      </c>
+      <c r="M35" s="112">
+        <f>SUM(I35:J35)/((1+'Project Details'!$F$6)^(B35/12))</f>
+        <v>4202.3544868745412</v>
+      </c>
+      <c r="N35" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K35)</f>
-        <v>-6646.2622407178569</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.2">
+        <v>30356.338146942726</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A36" s="115">
         <f>(1+'Project Details'!$F$5)^(B36/12)</f>
         <v>1.1023791513384635</v>
@@ -9058,23 +10860,31 @@
         <v>-4026.4295540699213</v>
       </c>
       <c r="I36" s="33">
-        <f>IF(MOD(B36,12)=0,Revenue!$E$8*A36,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J36" s="119">
         <f>IF(MOD(B36,12)=0,Revenue!$E$4*A36,0)</f>
         <v>0</v>
       </c>
       <c r="K36" s="112">
-        <f t="shared" si="0"/>
-        <v>-16967.310697051686</v>
-      </c>
-      <c r="L36" s="12">
+        <f>SUM(C36:J36)</f>
+        <v>-11774.433984722918</v>
+      </c>
+      <c r="L36" s="112">
+        <f>SUM(C36:H36)/((1+'Project Details'!$F$6)^(B36/12))</f>
+        <v>-13643.078310185963</v>
+      </c>
+      <c r="M36" s="112">
+        <f>SUM(I36:J36)/((1+'Project Details'!$F$6)^(B36/12))</f>
+        <v>4175.4892632309165</v>
+      </c>
+      <c r="N36" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K36)</f>
-        <v>-20289.340550903842</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.2">
+        <v>20888.749099987668</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A37" s="115">
         <f>(1+'Project Details'!$F$5)^(B37/12)</f>
         <v>1.1055439702319778</v>
@@ -9107,23 +10917,31 @@
         <v>-4037.9890255191526</v>
       </c>
       <c r="I37" s="33">
-        <f>IF(MOD(B37,12)=0,Revenue!$E$8*A37,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J37" s="119">
         <f>IF(MOD(B37,12)=0,Revenue!$E$4*A37,0)</f>
         <v>0</v>
       </c>
       <c r="K37" s="112">
-        <f t="shared" si="0"/>
-        <v>-16996.853518119955</v>
-      </c>
-      <c r="L37" s="12">
+        <f>SUM(C37:J37)</f>
+        <v>-11803.976805791188</v>
+      </c>
+      <c r="L37" s="112">
+        <f>SUM(C37:H37)/((1+'Project Details'!$F$6)^(B37/12))</f>
+        <v>-13579.462436994212</v>
+      </c>
+      <c r="M37" s="112">
+        <f>SUM(I37:J37)/((1+'Project Details'!$F$6)^(B37/12))</f>
+        <v>4148.7957862221092</v>
+      </c>
+      <c r="N37" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K37)</f>
-        <v>-33868.80298789806</v>
-      </c>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.2">
+        <v>11458.082449215552</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A38" s="115">
         <f>(1+'Project Details'!$F$5)^(B38/12)</f>
         <v>1.1087178749999997</v>
@@ -9156,23 +10974,31 @@
         <v>-4049.5816830401614</v>
       </c>
       <c r="I38" s="33">
-        <f>IF(MOD(B38,12)=0,Revenue!$E$8*A38,0)</f>
-        <v>69089.222803561628</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J38" s="119">
         <f>IF(MOD(B38,12)=0,Revenue!$E$4*A38,0)</f>
         <v>172427.80391999995</v>
       </c>
       <c r="K38" s="112">
-        <f t="shared" si="0"/>
-        <v>221718.75088242619</v>
-      </c>
-      <c r="L38" s="12">
+        <f>SUM(C38:J38)</f>
+        <v>157822.40479119332</v>
+      </c>
+      <c r="L38" s="112">
+        <f>SUM(C38:H38)/((1+'Project Details'!$F$6)^(B38/12))</f>
+        <v>-15716.509679303987</v>
+      </c>
+      <c r="M38" s="112">
+        <f>SUM(I38:J38)/((1+'Project Details'!$F$6)^(B38/12))</f>
+        <v>141001.02295788933</v>
+      </c>
+      <c r="N38" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K38)</f>
-        <v>142138.68990129122</v>
-      </c>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.2">
+        <v>136742.59572780103</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A39" s="115">
         <f>(1+'Project Details'!$F$5)^(B39/12)</f>
         <v>1.1119008917271547</v>
@@ -9205,23 +11031,31 @@
         <v>-4061.2076219067976</v>
       </c>
       <c r="I39" s="33">
-        <f>IF(MOD(B39,12)=0,Revenue!$E$8*A39,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J39" s="119">
         <f>IF(MOD(B39,12)=0,Revenue!$E$4*A39,0)</f>
         <v>0</v>
       </c>
       <c r="K39" s="112">
-        <f t="shared" si="0"/>
-        <v>-10379.326651917258</v>
-      </c>
-      <c r="L39" s="12">
+        <f>SUM(C39:J39)</f>
+        <v>-5186.4499395884905</v>
+      </c>
+      <c r="L39" s="112">
+        <f>SUM(C39:H39)/((1+'Project Details'!$F$6)^(B39/12))</f>
+        <v>-8186.7702103348747</v>
+      </c>
+      <c r="M39" s="112">
+        <f>SUM(I39:J39)/((1+'Project Details'!$F$6)^(B39/12))</f>
+        <v>4095.9196872931948</v>
+      </c>
+      <c r="N39" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K39)</f>
-        <v>133951.91969095633</v>
-      </c>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.2">
+        <v>132651.74520475935</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A40" s="115">
         <f>(1+'Project Details'!$F$5)^(B40/12)</f>
         <v>1.1150930465729543</v>
@@ -9254,23 +11088,31 @@
         <v>-4072.8669376664338</v>
       </c>
       <c r="I40" s="33">
-        <f>IF(MOD(B40,12)=0,Revenue!$E$8*A40,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J40" s="119">
         <f>IF(MOD(B40,12)=0,Revenue!$E$4*A40,0)</f>
         <v>0</v>
       </c>
       <c r="K40" s="112">
-        <f t="shared" si="0"/>
-        <v>-10409.124647507124</v>
-      </c>
-      <c r="L40" s="12">
+        <f>SUM(C40:J40)</f>
+        <v>-5216.2479351783568</v>
+      </c>
+      <c r="L40" s="112">
+        <f>SUM(C40:H40)/((1+'Project Details'!$F$6)^(B40/12))</f>
+        <v>-8157.7861566820375</v>
+      </c>
+      <c r="M40" s="112">
+        <f>SUM(I40:J40)/((1+'Project Details'!$F$6)^(B40/12))</f>
+        <v>4069.7348904681908</v>
+      </c>
+      <c r="N40" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K40)</f>
-        <v>125794.13353427428</v>
-      </c>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.2">
+        <v>128563.69393854549</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A41" s="115">
         <f>(1+'Project Details'!$F$5)^(B41/12)</f>
         <v>1.1182943657720117</v>
@@ -9303,23 +11145,31 @@
         <v>-4084.5597261407497</v>
       </c>
       <c r="I41" s="33">
-        <f>IF(MOD(B41,12)=0,Revenue!$E$8*A41,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J41" s="119">
         <f>IF(MOD(B41,12)=0,Revenue!$E$4*A41,0)</f>
         <v>0</v>
       </c>
       <c r="K41" s="112">
-        <f t="shared" si="0"/>
-        <v>-10439.008190124361</v>
-      </c>
-      <c r="L41" s="12">
+        <f>SUM(C41:J41)</f>
+        <v>-5246.131477795594</v>
+      </c>
+      <c r="L41" s="112">
+        <f>SUM(C41:H41)/((1+'Project Details'!$F$6)^(B41/12))</f>
+        <v>-8128.9047168005145</v>
+      </c>
+      <c r="M41" s="112">
+        <f>SUM(I41:J41)/((1+'Project Details'!$F$6)^(B41/12))</f>
+        <v>4043.7174903787468</v>
+      </c>
+      <c r="N41" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K41)</f>
-        <v>117665.22881747375</v>
-      </c>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.2">
+        <v>124478.50671212372</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A42" s="115">
         <f>(1+'Project Details'!$F$5)^(B42/12)</f>
         <v>1.1215048756342572</v>
@@ -9352,23 +11202,31 @@
         <v>-4096.2860834265193</v>
       </c>
       <c r="I42" s="33">
-        <f>IF(MOD(B42,12)=0,Revenue!$E$8*A42,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J42" s="119">
         <f>IF(MOD(B42,12)=0,Revenue!$E$4*A42,0)</f>
         <v>0</v>
       </c>
       <c r="K42" s="112">
-        <f t="shared" si="0"/>
-        <v>-10468.977525365819</v>
-      </c>
-      <c r="L42" s="12">
+        <f>SUM(C42:J42)</f>
+        <v>-5276.1008130370519</v>
+      </c>
+      <c r="L42" s="112">
+        <f>SUM(C42:H42)/((1+'Project Details'!$F$6)^(B42/12))</f>
+        <v>-8100.1255274013638</v>
+      </c>
+      <c r="M42" s="112">
+        <f>SUM(I42:J42)/((1+'Project Details'!$F$6)^(B42/12))</f>
+        <v>4017.8664168746031</v>
+      </c>
+      <c r="N42" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K42)</f>
-        <v>109565.10329007238</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.2">
+        <v>120396.24760159696</v>
+      </c>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A43" s="115">
         <f>(1+'Project Details'!$F$5)^(B43/12)</f>
         <v>1.1247246025451538</v>
@@ -9401,23 +11259,31 @@
         <v>-4108.0461058964001</v>
       </c>
       <c r="I43" s="33">
-        <f>IF(MOD(B43,12)=0,Revenue!$E$8*A43,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J43" s="119">
         <f>IF(MOD(B43,12)=0,Revenue!$E$4*A43,0)</f>
         <v>0</v>
       </c>
       <c r="K43" s="112">
-        <f t="shared" si="0"/>
-        <v>-10499.032899533435</v>
-      </c>
-      <c r="L43" s="12">
+        <f>SUM(C43:J43)</f>
+        <v>-5306.1561872046677</v>
+      </c>
+      <c r="L43" s="112">
+        <f>SUM(C43:H43)/((1+'Project Details'!$F$6)^(B43/12))</f>
+        <v>-8071.4482264818234</v>
+      </c>
+      <c r="M43" s="112">
+        <f>SUM(I43:J43)/((1+'Project Details'!$F$6)^(B43/12))</f>
+        <v>3992.1806066468657</v>
+      </c>
+      <c r="N43" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K43)</f>
-        <v>101493.65506359056</v>
-      </c>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.2">
+        <v>116316.97998176198</v>
+      </c>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A44" s="115">
         <f>(1+'Project Details'!$F$5)^(B44/12)</f>
         <v>1.1279535729659147</v>
@@ -9450,23 +11316,31 @@
         <v>-4119.8398901997261</v>
       </c>
       <c r="I44" s="33">
-        <f>IF(MOD(B44,12)=0,Revenue!$E$8*A44,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J44" s="119">
         <f>IF(MOD(B44,12)=0,Revenue!$E$4*A44,0)</f>
         <v>0</v>
       </c>
       <c r="K44" s="112">
-        <f t="shared" si="0"/>
-        <v>-10529.174559636249</v>
-      </c>
-      <c r="L44" s="12">
+        <f>SUM(C44:J44)</f>
+        <v>-5336.2978473074818</v>
+      </c>
+      <c r="L44" s="112">
+        <f>SUM(C44:H44)/((1+'Project Details'!$F$6)^(B44/12))</f>
+        <v>-8042.8724533207396</v>
+      </c>
+      <c r="M44" s="112">
+        <f>SUM(I44:J44)/((1+'Project Details'!$F$6)^(B44/12))</f>
+        <v>3966.6590031842616</v>
+      </c>
+      <c r="N44" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K44)</f>
-        <v>93450.782610269802</v>
-      </c>
-    </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.2">
+        <v>112240.7665316255</v>
+      </c>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A45" s="115">
         <f>(1+'Project Details'!$F$5)^(B45/12)</f>
         <v>1.1311918134337204</v>
@@ -9499,23 +11373,31 @@
         <v>-4131.6675332633013</v>
       </c>
       <c r="I45" s="33">
-        <f>IF(MOD(B45,12)=0,Revenue!$E$8*A45,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J45" s="119">
         <f>IF(MOD(B45,12)=0,Revenue!$E$4*A45,0)</f>
         <v>0</v>
       </c>
       <c r="K45" s="112">
-        <f t="shared" si="0"/>
-        <v>-10559.402753392442</v>
-      </c>
-      <c r="L45" s="12">
+        <f>SUM(C45:J45)</f>
+        <v>-5366.5260410636747</v>
+      </c>
+      <c r="L45" s="112">
+        <f>SUM(C45:H45)/((1+'Project Details'!$F$6)^(B45/12))</f>
+        <v>-8014.3978484740455</v>
+      </c>
+      <c r="M45" s="112">
+        <f>SUM(I45:J45)/((1+'Project Details'!$F$6)^(B45/12))</f>
+        <v>3941.3005567296896</v>
+      </c>
+      <c r="N45" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K45)</f>
-        <v>85436.384761795736</v>
-      </c>
-    </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.2">
+        <v>108167.66923988114</v>
+      </c>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A46" s="115">
         <f>(1+'Project Details'!$F$5)^(B46/12)</f>
         <v>1.1344393505619372</v>
@@ -9548,23 +11430,31 @@
         <v>-4143.5291322921967</v>
       </c>
       <c r="I46" s="33">
-        <f>IF(MOD(B46,12)=0,Revenue!$E$8*A46,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J46" s="119">
         <f>IF(MOD(B46,12)=0,Revenue!$E$4*A46,0)</f>
         <v>0</v>
       </c>
       <c r="K46" s="112">
-        <f t="shared" si="0"/>
-        <v>-10589.717729231372</v>
-      </c>
-      <c r="L46" s="12">
+        <f>SUM(C46:J46)</f>
+        <v>-5396.8410169026047</v>
+      </c>
+      <c r="L46" s="112">
+        <f>SUM(C46:H46)/((1+'Project Details'!$F$6)^(B46/12))</f>
+        <v>-7986.0240537702321</v>
+      </c>
+      <c r="M46" s="112">
+        <f>SUM(I46:J46)/((1+'Project Details'!$F$6)^(B46/12))</f>
+        <v>3916.1042242370368</v>
+      </c>
+      <c r="N46" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K46)</f>
-        <v>77450.360708025502</v>
-      </c>
-    </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.2">
+        <v>104097.74941034794</v>
+      </c>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A47" s="115">
         <f>(1+'Project Details'!$F$5)^(B47/12)</f>
         <v>1.1376962110403357</v>
@@ -9597,23 +11487,31 @@
         <v>-4155.4247847705519</v>
       </c>
       <c r="I47" s="33">
-        <f>IF(MOD(B47,12)=0,Revenue!$E$8*A47,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J47" s="119">
         <f>IF(MOD(B47,12)=0,Revenue!$E$4*A47,0)</f>
         <v>0</v>
       </c>
       <c r="K47" s="112">
-        <f t="shared" si="0"/>
-        <v>-10620.119736295606</v>
-      </c>
-      <c r="L47" s="12">
+        <f>SUM(C47:J47)</f>
+        <v>-5427.2430239668392</v>
+      </c>
+      <c r="L47" s="112">
+        <f>SUM(C47:H47)/((1+'Project Details'!$F$6)^(B47/12))</f>
+        <v>-7957.7507123058394</v>
+      </c>
+      <c r="M47" s="112">
+        <f>SUM(I47:J47)/((1+'Project Details'!$F$6)^(B47/12))</f>
+        <v>3891.0689693282784</v>
+      </c>
+      <c r="N47" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K47)</f>
-        <v>69492.609995719657</v>
-      </c>
-    </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.2">
+        <v>100031.06766737037</v>
+      </c>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A48" s="115">
         <f>(1+'Project Details'!$F$5)^(B48/12)</f>
         <v>1.1409624216353096</v>
@@ -9646,23 +11544,31 @@
         <v>-4167.3545884623682</v>
       </c>
       <c r="I48" s="33">
-        <f>IF(MOD(B48,12)=0,Revenue!$E$8*A48,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J48" s="119">
         <f>IF(MOD(B48,12)=0,Revenue!$E$4*A48,0)</f>
         <v>0</v>
       </c>
       <c r="K48" s="112">
-        <f t="shared" si="0"/>
-        <v>-10650.609024442976</v>
-      </c>
-      <c r="L48" s="12">
+        <f>SUM(C48:J48)</f>
+        <v>-5457.732312114209</v>
+      </c>
+      <c r="L48" s="112">
+        <f>SUM(C48:H48)/((1+'Project Details'!$F$6)^(B48/12))</f>
+        <v>-7929.5774684409744</v>
+      </c>
+      <c r="M48" s="112">
+        <f>SUM(I48:J48)/((1+'Project Details'!$F$6)^(B48/12))</f>
+        <v>3866.1937622508494</v>
+      </c>
+      <c r="N48" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K48)</f>
-        <v>61563.032527278665</v>
-      </c>
-    </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.2">
+        <v>95967.683961180242</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A49" s="115">
         <f>(1+'Project Details'!$F$5)^(B49/12)</f>
         <v>1.144238009190097</v>
@@ -9695,23 +11601,31 @@
         <v>-4179.3186414123229</v>
       </c>
       <c r="I49" s="33">
-        <f>IF(MOD(B49,12)=0,Revenue!$E$8*A49,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J49" s="119">
         <f>IF(MOD(B49,12)=0,Revenue!$E$4*A49,0)</f>
         <v>0</v>
       </c>
       <c r="K49" s="112">
-        <f t="shared" si="0"/>
-        <v>-10681.185844248634</v>
-      </c>
-      <c r="L49" s="12">
+        <f>SUM(C49:J49)</f>
+        <v>-5488.3091319198666</v>
+      </c>
+      <c r="L49" s="112">
+        <f>SUM(C49:H49)/((1+'Project Details'!$F$6)^(B49/12))</f>
+        <v>-7901.5039677948353</v>
+      </c>
+      <c r="M49" s="112">
+        <f>SUM(I49:J49)/((1+'Project Details'!$F$6)^(B49/12))</f>
+        <v>3841.4775798352857</v>
+      </c>
+      <c r="N49" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K49)</f>
-        <v>53661.528559483821</v>
-      </c>
-    </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.2">
+        <v>91907.657573220684</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A50" s="115">
         <f>(1+'Project Details'!$F$5)^(B50/12)</f>
         <v>1.1475230006249997</v>
@@ -9744,23 +11658,31 @@
         <v>-4191.3170419465669</v>
       </c>
       <c r="I50" s="33">
-        <f>IF(MOD(B50,12)=0,Revenue!$E$8*A50,0)</f>
-        <v>71507.345601686276</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J50" s="119">
         <f>IF(MOD(B50,12)=0,Revenue!$E$4*A50,0)</f>
         <v>178462.77705719994</v>
       </c>
       <c r="K50" s="112">
-        <f t="shared" si="0"/>
-        <v>236389.46471031662</v>
-      </c>
-      <c r="L50" s="12">
+        <f>SUM(C50:J50)</f>
+        <v>170074.9958209591</v>
+      </c>
+      <c r="L50" s="112">
+        <f>SUM(C50:H50)/((1+'Project Details'!$F$6)^(B50/12))</f>
+        <v>-9982.1890128161031</v>
+      </c>
+      <c r="M50" s="112">
+        <f>SUM(I50:J50)/((1+'Project Details'!$F$6)^(B50/12))</f>
+        <v>134992.38815545305</v>
+      </c>
+      <c r="N50" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K50)</f>
-        <v>227414.84200814046</v>
-      </c>
-    </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.2">
+        <v>216917.85671585784</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A51" s="115">
         <f>(1+'Project Details'!$F$5)^(B51/12)</f>
         <v>1.1508174229376049</v>
@@ -9793,23 +11715,31 @@
         <v>-4203.3498886735351</v>
       </c>
       <c r="I51" s="33">
-        <f>IF(MOD(B51,12)=0,Revenue!$E$8*A51,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J51" s="119">
         <f>IF(MOD(B51,12)=0,Revenue!$E$4*A51,0)</f>
         <v>0</v>
       </c>
       <c r="K51" s="112">
-        <f t="shared" si="0"/>
-        <v>-10742.603084734361</v>
-      </c>
-      <c r="L51" s="12">
+        <f>SUM(C51:J51)</f>
+        <v>-5549.7263724055938</v>
+      </c>
+      <c r="L51" s="112">
+        <f>SUM(C51:H51)/((1+'Project Details'!$F$6)^(B51/12))</f>
+        <v>-7845.6547849042554</v>
+      </c>
+      <c r="M51" s="112">
+        <f>SUM(I51:J51)/((1+'Project Details'!$F$6)^(B51/12))</f>
+        <v>3792.5182289751806</v>
+      </c>
+      <c r="N51" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K51)</f>
-        <v>219569.18722323619</v>
-      </c>
-    </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.2">
+        <v>212864.72015992875</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A52" s="115">
         <f>(1+'Project Details'!$F$5)^(B52/12)</f>
         <v>1.1541213032030075</v>
@@ -9842,23 +11772,31 @@
         <v>-4215.4172804847585</v>
       </c>
       <c r="I52" s="33">
-        <f>IF(MOD(B52,12)=0,Revenue!$E$8*A52,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J52" s="119">
         <f>IF(MOD(B52,12)=0,Revenue!$E$4*A52,0)</f>
         <v>0</v>
       </c>
       <c r="K52" s="112">
-        <f t="shared" si="0"/>
-        <v>-10773.444010169873</v>
-      </c>
-      <c r="L52" s="12">
+        <f>SUM(C52:J52)</f>
+        <v>-5580.5672978411058</v>
+      </c>
+      <c r="L52" s="112">
+        <f>SUM(C52:H52)/((1+'Project Details'!$F$6)^(B52/12))</f>
+        <v>-7817.8784001536187</v>
+      </c>
+      <c r="M52" s="112">
+        <f>SUM(I52:J52)/((1+'Project Details'!$F$6)^(B52/12))</f>
+        <v>3768.2730467298061</v>
+      </c>
+      <c r="N52" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K52)</f>
-        <v>211751.30882308257</v>
-      </c>
-    </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.2">
+        <v>208815.11480650492</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A53" s="115">
         <f>(1+'Project Details'!$F$5)^(B53/12)</f>
         <v>1.157434668574032</v>
@@ -9891,23 +11829,31 @@
         <v>-4227.5193165556757</v>
       </c>
       <c r="I53" s="33">
-        <f>IF(MOD(B53,12)=0,Revenue!$E$8*A53,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J53" s="119">
         <f>IF(MOD(B53,12)=0,Revenue!$E$4*A53,0)</f>
         <v>0</v>
       </c>
       <c r="K53" s="112">
-        <f t="shared" si="0"/>
-        <v>-10804.373476778714</v>
-      </c>
-      <c r="L53" s="12">
+        <f>SUM(C53:J53)</f>
+        <v>-5611.4967644499466</v>
+      </c>
+      <c r="L53" s="112">
+        <f>SUM(C53:H53)/((1+'Project Details'!$F$6)^(B53/12))</f>
+        <v>-7790.2003536004931</v>
+      </c>
+      <c r="M53" s="112">
+        <f>SUM(I53:J53)/((1+'Project Details'!$F$6)^(B53/12))</f>
+        <v>3744.1828614618025</v>
+      </c>
+      <c r="N53" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K53)</f>
-        <v>203961.10846948205</v>
-      </c>
-    </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.2">
+        <v>204769.09731436623</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A54" s="115">
         <f>(1+'Project Details'!$F$5)^(B54/12)</f>
         <v>1.1607575462814561</v>
@@ -9940,23 +11886,31 @@
         <v>-4239.6560963464472</v>
       </c>
       <c r="I54" s="33">
-        <f>IF(MOD(B54,12)=0,Revenue!$E$8*A54,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J54" s="119">
         <f>IF(MOD(B54,12)=0,Revenue!$E$4*A54,0)</f>
         <v>0</v>
       </c>
       <c r="K54" s="112">
-        <f t="shared" si="0"/>
-        <v>-10835.391738753622</v>
-      </c>
-      <c r="L54" s="12">
+        <f>SUM(C54:J54)</f>
+        <v>-5642.515026424855</v>
+      </c>
+      <c r="L54" s="112">
+        <f>SUM(C54:H54)/((1+'Project Details'!$F$6)^(B54/12))</f>
+        <v>-7762.6202970929735</v>
+      </c>
+      <c r="M54" s="112">
+        <f>SUM(I54:J54)/((1+'Project Details'!$F$6)^(B54/12))</f>
+        <v>3720.2466822912997</v>
+      </c>
+      <c r="N54" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K54)</f>
-        <v>196198.48817238907</v>
-      </c>
-    </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.2">
+        <v>200726.72369956452</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A55" s="115">
         <f>(1+'Project Details'!$F$5)^(B55/12)</f>
         <v>1.1640899636342341</v>
@@ -9989,23 +11943,31 @@
         <v>-4251.8277196027739</v>
       </c>
       <c r="I55" s="33">
-        <f>IF(MOD(B55,12)=0,Revenue!$E$8*A55,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J55" s="119">
         <f>IF(MOD(B55,12)=0,Revenue!$E$4*A55,0)</f>
         <v>0</v>
       </c>
       <c r="K55" s="112">
-        <f t="shared" si="0"/>
-        <v>-10866.499051017105</v>
-      </c>
-      <c r="L55" s="12">
+        <f>SUM(C55:J55)</f>
+        <v>-5673.6223386883375</v>
+      </c>
+      <c r="L55" s="112">
+        <f>SUM(C55:H55)/((1+'Project Details'!$F$6)^(B55/12))</f>
+        <v>-7735.1378837117463</v>
+      </c>
+      <c r="M55" s="112">
+        <f>SUM(I55:J55)/((1+'Project Details'!$F$6)^(B55/12))</f>
+        <v>3696.4635246730236</v>
+      </c>
+      <c r="N55" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K55)</f>
-        <v>188463.35028867732</v>
-      </c>
-    </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.2">
+        <v>196688.04934052582</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A56" s="115">
         <f>(1+'Project Details'!$F$5)^(B56/12)</f>
         <v>1.1674319480197215</v>
@@ -10038,23 +12000,31 @@
         <v>-4264.0342863567157</v>
       </c>
       <c r="I56" s="33">
-        <f>IF(MOD(B56,12)=0,Revenue!$E$8*A56,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J56" s="119">
         <f>IF(MOD(B56,12)=0,Revenue!$E$4*A56,0)</f>
         <v>0</v>
       </c>
       <c r="K56" s="112">
-        <f t="shared" si="0"/>
-        <v>-10897.695669223516</v>
-      </c>
-      <c r="L56" s="12">
+        <f>SUM(C56:J56)</f>
+        <v>-5704.8189568947491</v>
+      </c>
+      <c r="L56" s="112">
+        <f>SUM(C56:H56)/((1+'Project Details'!$F$6)^(B56/12))</f>
+        <v>-7707.752767765709</v>
+      </c>
+      <c r="M56" s="112">
+        <f>SUM(I56:J56)/((1+'Project Details'!$F$6)^(B56/12))</f>
+        <v>3672.8324103557979</v>
+      </c>
+      <c r="N56" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K56)</f>
-        <v>180755.5975209116</v>
-      </c>
-    </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.2">
+        <v>192653.12898311589</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A57" s="115">
         <f>(1+'Project Details'!$F$5)^(B57/12)</f>
         <v>1.1707835269039004</v>
@@ -10087,23 +12057,31 @@
         <v>-4276.2758969275155</v>
       </c>
       <c r="I57" s="33">
-        <f>IF(MOD(B57,12)=0,Revenue!$E$8*A57,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J57" s="119">
         <f>IF(MOD(B57,12)=0,Revenue!$E$4*A57,0)</f>
         <v>0</v>
       </c>
       <c r="K57" s="112">
-        <f t="shared" si="0"/>
-        <v>-10928.981849761178</v>
-      </c>
-      <c r="L57" s="12">
+        <f>SUM(C57:J57)</f>
+        <v>-5736.1051374324106</v>
+      </c>
+      <c r="L57" s="112">
+        <f>SUM(C57:H57)/((1+'Project Details'!$F$6)^(B57/12))</f>
+        <v>-7680.4646047876276</v>
+      </c>
+      <c r="M57" s="112">
+        <f>SUM(I57:J57)/((1+'Project Details'!$F$6)^(B57/12))</f>
+        <v>3649.3523673423056</v>
+      </c>
+      <c r="N57" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K57)</f>
-        <v>173075.13291612396</v>
-      </c>
-    </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.2">
+        <v>188622.01674567058</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A58" s="115">
         <f>(1+'Project Details'!$F$5)^(B58/12)</f>
         <v>1.1741447278316048</v>
@@ -10136,23 +12114,31 @@
         <v>-4288.5526519224231</v>
       </c>
       <c r="I58" s="33">
-        <f>IF(MOD(B58,12)=0,Revenue!$E$8*A58,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J58" s="119">
         <f>IF(MOD(B58,12)=0,Revenue!$E$4*A58,0)</f>
         <v>0</v>
       </c>
       <c r="K58" s="112">
-        <f t="shared" si="0"/>
-        <v>-10960.357849754468</v>
-      </c>
-      <c r="L58" s="12">
+        <f>SUM(C58:J58)</f>
+        <v>-5767.4811374257006</v>
+      </c>
+      <c r="L58" s="112">
+        <f>SUM(C58:H58)/((1+'Project Details'!$F$6)^(B58/12))</f>
+        <v>-7653.2730515298035</v>
+      </c>
+      <c r="M58" s="112">
+        <f>SUM(I58:J58)/((1+'Project Details'!$F$6)^(B58/12))</f>
+        <v>3626.0224298491075</v>
+      </c>
+      <c r="N58" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K58)</f>
-        <v>165421.85986459412</v>
-      </c>
-    </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.2">
+        <v>184594.76612398989</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A59" s="115">
         <f>(1+'Project Details'!$F$5)^(B59/12)</f>
         <v>1.1775155784267473</v>
@@ -10185,23 +12171,31 @@
         <v>-4300.8646522375202</v>
       </c>
       <c r="I59" s="33">
-        <f>IF(MOD(B59,12)=0,Revenue!$E$8*A59,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J59" s="119">
         <f>IF(MOD(B59,12)=0,Revenue!$E$4*A59,0)</f>
         <v>0</v>
       </c>
       <c r="K59" s="112">
-        <f t="shared" si="0"/>
-        <v>-10991.823927065951</v>
-      </c>
-      <c r="L59" s="12">
+        <f>SUM(C59:J59)</f>
+        <v>-5798.9472147371835</v>
+      </c>
+      <c r="L59" s="112">
+        <f>SUM(C59:H59)/((1+'Project Details'!$F$6)^(B59/12))</f>
+        <v>-7626.177765959761</v>
+      </c>
+      <c r="M59" s="112">
+        <f>SUM(I59:J59)/((1+'Project Details'!$F$6)^(B59/12))</f>
+        <v>3602.8416382669243</v>
+      </c>
+      <c r="N59" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K59)</f>
-        <v>157795.68209863434</v>
-      </c>
-    </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.2">
+        <v>180571.42999629703</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A60" s="115">
         <f>(1+'Project Details'!$F$5)^(B60/12)</f>
         <v>1.1808961063925454</v>
@@ -10234,23 +12228,31 @@
         <v>-4313.2119990585506</v>
       </c>
       <c r="I60" s="33">
-        <f>IF(MOD(B60,12)=0,Revenue!$E$8*A60,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J60" s="119">
         <f>IF(MOD(B60,12)=0,Revenue!$E$4*A60,0)</f>
         <v>0</v>
       </c>
       <c r="K60" s="112">
-        <f t="shared" si="0"/>
-        <v>-11023.380340298478</v>
-      </c>
-      <c r="L60" s="12">
+        <f>SUM(C60:J60)</f>
+        <v>-5830.5036279697106</v>
+      </c>
+      <c r="L60" s="112">
+        <f>SUM(C60:H60)/((1+'Project Details'!$F$6)^(B60/12))</f>
+        <v>-7599.1784072559312</v>
+      </c>
+      <c r="M60" s="112">
+        <f>SUM(I60:J60)/((1+'Project Details'!$F$6)^(B60/12))</f>
+        <v>3579.8090391211563</v>
+      </c>
+      <c r="N60" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K60)</f>
-        <v>150196.5036913784</v>
-      </c>
-    </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.2">
+        <v>176552.06062816223</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A61" s="115">
         <f>(1+'Project Details'!$F$5)^(B61/12)</f>
         <v>1.1842863395117502</v>
@@ -10283,23 +12285,31 @@
         <v>-4325.5947938617537</v>
       </c>
       <c r="I61" s="33">
-        <f>IF(MOD(B61,12)=0,Revenue!$E$8*A61,0)</f>
-        <v>0</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J61" s="119">
         <f>IF(MOD(B61,12)=0,Revenue!$E$4*A61,0)</f>
         <v>0</v>
       </c>
       <c r="K61" s="112">
-        <f t="shared" si="0"/>
-        <v>-11055.027348797335</v>
-      </c>
-      <c r="L61" s="12">
+        <f>SUM(C61:J61)</f>
+        <v>-5862.1506364685683</v>
+      </c>
+      <c r="L61" s="112">
+        <f>SUM(C61:H61)/((1+'Project Details'!$F$6)^(B61/12))</f>
+        <v>-7572.2746358033828</v>
+      </c>
+      <c r="M61" s="112">
+        <f>SUM(I61:J61)/((1+'Project Details'!$F$6)^(B61/12))</f>
+        <v>3556.9236850326715</v>
+      </c>
+      <c r="N61" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K61)</f>
-        <v>142624.22905557498</v>
-      </c>
-    </row>
-    <row r="62" spans="1:12" x14ac:dyDescent="0.2">
+        <v>172536.70967739151</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A62" s="115">
         <f>(1+'Project Details'!$F$5)^(B62/12)</f>
         <v>1.1876863056468745</v>
@@ -10331,470 +12341,151 @@
         <v>-4338.0131384146962</v>
       </c>
       <c r="I62" s="33">
-        <f>IF(MOD(B62,12)=0,Revenue!$E$8*A62,0)</f>
-        <v>74010.102697745286</v>
+        <f>Revenue!$E$8/12</f>
+        <v>5192.8767123287671</v>
       </c>
       <c r="J62" s="119">
         <v>0</v>
       </c>
       <c r="K62" s="112">
-        <f t="shared" si="0"/>
-        <v>62923.337485092932</v>
-      </c>
-      <c r="L62" s="12">
+        <f>SUM(C62:J62)</f>
+        <v>-5893.8885003235882</v>
+      </c>
+      <c r="L62" s="112">
+        <f>SUM(C62:H62)/((1+'Project Details'!$F$6)^(B62/12))</f>
+        <v>-7545.4661131895364</v>
+      </c>
+      <c r="M62" s="112">
+        <f>SUM(I62:J62)/((1+'Project Details'!$F$6)^(B62/12))</f>
+        <v>3534.184634678837</v>
+      </c>
+      <c r="N62" s="12">
         <f>$K$2+NPV((1+'Project Details'!$F$6)^(1/12)-1,$K$3:K62)</f>
-        <v>185448.79524921341</v>
+        <v>168525.42819888081</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="O4:P4"/>
+    <mergeCell ref="Q4:R4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9ECABA95-71D1-0E46-8056-8FE7EC645263}">
-  <dimension ref="A1:M18"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FD8A865-E1FD-4B4B-89C0-66964BC64EB8}">
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
-    <col min="2" max="2" width="19.6640625" customWidth="1"/>
-    <col min="3" max="3" width="16.6640625" customWidth="1"/>
-    <col min="4" max="11" width="14.33203125" customWidth="1"/>
+    <col min="2" max="2" width="18.33203125" customWidth="1"/>
+    <col min="3" max="3" width="17.33203125" customWidth="1"/>
+    <col min="4" max="4" width="26.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B1" s="147"/>
-      <c r="C1" s="147"/>
-    </row>
-    <row r="2" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="M2" s="120"/>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B3" s="126">
-        <v>0.12</v>
-      </c>
-      <c r="C3" s="125" t="s">
-        <v>182</v>
-      </c>
-      <c r="D3" s="171" t="s">
-        <v>208</v>
-      </c>
-      <c r="E3" s="172"/>
-      <c r="F3" s="172"/>
-      <c r="G3" s="172"/>
-      <c r="H3" s="172"/>
-      <c r="I3" s="172"/>
-      <c r="J3" s="172"/>
-      <c r="K3" s="172"/>
-    </row>
-    <row r="4" spans="1:13" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="10"/>
-      <c r="B4" s="127">
-        <v>180</v>
-      </c>
-      <c r="C4" s="127">
-        <f>Cashflow!P5</f>
-        <v>185448.79524921341</v>
-      </c>
-      <c r="D4" s="123">
-        <v>180</v>
-      </c>
-      <c r="E4" s="12">
-        <f>D4+10</f>
-        <v>190</v>
-      </c>
-      <c r="F4" s="12">
-        <f t="shared" ref="F4:J4" si="0">E4+10</f>
-        <v>200</v>
-      </c>
-      <c r="G4" s="12">
+    <row r="1" spans="1:4" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="173" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="173" t="s">
+        <v>212</v>
+      </c>
+      <c r="C1" s="173" t="s">
+        <v>213</v>
+      </c>
+      <c r="D1" s="173" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="174">
+        <f>SUM(Cashflow!M2:M13)</f>
+        <v>210496.63225562812</v>
+      </c>
+      <c r="C2" s="174">
+        <f>ABS(SUM(Cashflow!L2:L13))</f>
+        <v>249372.7018597956</v>
+      </c>
+      <c r="D2" s="174">
+        <f>B2-C2</f>
+        <v>-38876.069604167482</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
+        <f>1+A2</f>
+        <v>2</v>
+      </c>
+      <c r="B3" s="174">
+        <f>SUM(Cashflow!M14:M25)</f>
+        <v>204752.50830366375</v>
+      </c>
+      <c r="C3" s="174">
+        <f>ABS(SUM(Cashflow!L14:L25))</f>
+        <v>179313.43397986534</v>
+      </c>
+      <c r="D3" s="174">
+        <f>B3-C3+D2</f>
+        <v>-13436.995280369068</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="1">
+        <f t="shared" ref="A4:A7" si="0">1+A3</f>
+        <v>3</v>
+      </c>
+      <c r="B4" s="174">
+        <f>SUM(Cashflow!M26:M37)</f>
+        <v>194415.65583672572</v>
+      </c>
+      <c r="C4" s="174">
+        <f>ABS(SUM(Cashflow!L26:L37))</f>
+        <v>169520.57810714102</v>
+      </c>
+      <c r="D4" s="174">
+        <f t="shared" ref="D4:D6" si="1">B4-C4+D3</f>
+        <v>11458.082449215639</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="1">
         <f t="shared" si="0"/>
-        <v>210</v>
-      </c>
-      <c r="H4" s="12">
+        <v>4</v>
+      </c>
+      <c r="B5" s="174">
+        <f>SUM(Cashflow!M38:M49)</f>
+        <v>184643.24614511634</v>
+      </c>
+      <c r="C5" s="174">
+        <f>ABS(SUM(Cashflow!L38:L49))</f>
+        <v>104193.67102111128</v>
+      </c>
+      <c r="D5" s="174">
+        <f t="shared" si="1"/>
+        <v>91907.657573220698</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="1">
         <f t="shared" si="0"/>
-        <v>220</v>
-      </c>
-      <c r="I4" s="12">
-        <f t="shared" si="0"/>
-        <v>230</v>
-      </c>
-      <c r="J4" s="12">
-        <f t="shared" si="0"/>
-        <v>240</v>
-      </c>
-      <c r="K4" s="12">
-        <f>J4+10</f>
-        <v>250</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A5" s="10"/>
-      <c r="B5" s="169" t="s">
-        <v>196</v>
-      </c>
-      <c r="C5" s="124">
-        <v>0.1</v>
-      </c>
-      <c r="D5" s="12">
-        <f t="dataTable" ref="D5:K15" dt2D="1" dtr="1" r1="B4" r2="B3"/>
-        <v>67016.123779569025</v>
-      </c>
-      <c r="E5" s="12">
-        <v>100138.54131429124</v>
-      </c>
-      <c r="F5" s="12">
-        <v>133260.95884901349</v>
-      </c>
-      <c r="G5" s="12">
-        <v>166383.37638373568</v>
-      </c>
-      <c r="H5" s="12">
-        <v>199505.79391845793</v>
-      </c>
-      <c r="I5" s="12">
-        <v>232628.21145318018</v>
-      </c>
-      <c r="J5" s="12">
-        <v>265750.62898790243</v>
-      </c>
-      <c r="K5" s="12">
-        <v>298873.04652262456</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A6" s="10"/>
-      <c r="B6" s="170"/>
-      <c r="C6" s="122">
-        <f>C5+0.01</f>
-        <v>0.11</v>
-      </c>
-      <c r="D6" s="12">
-        <v>126232.45951439119</v>
-      </c>
-      <c r="E6" s="12">
-        <v>162667.1188025857</v>
-      </c>
-      <c r="F6" s="12">
-        <v>199101.77809078014</v>
-      </c>
-      <c r="G6" s="12">
-        <v>235536.43737897463</v>
-      </c>
-      <c r="H6" s="12">
-        <v>271971.09666716913</v>
-      </c>
-      <c r="I6" s="12">
-        <v>308405.75595536362</v>
-      </c>
-      <c r="J6" s="12">
-        <v>344840.415243558</v>
-      </c>
-      <c r="K6" s="12">
-        <v>381275.0745317525</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A7" s="10"/>
-      <c r="B7" s="170"/>
-      <c r="C7" s="122">
-        <f t="shared" ref="C7:C15" si="1">C6+0.01</f>
-        <v>0.12</v>
-      </c>
-      <c r="D7" s="12">
-        <v>185448.79524921341</v>
-      </c>
-      <c r="E7" s="12">
-        <v>225195.69629088012</v>
-      </c>
-      <c r="F7" s="12">
-        <v>264942.59733254684</v>
-      </c>
-      <c r="G7" s="12">
-        <v>304689.49837421346</v>
-      </c>
-      <c r="H7" s="12">
-        <v>344436.39941588009</v>
-      </c>
-      <c r="I7" s="12">
-        <v>384183.30045754684</v>
-      </c>
-      <c r="J7" s="12">
-        <v>423930.20149921358</v>
-      </c>
-      <c r="K7" s="12">
-        <v>463677.10254088021</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A8" s="10"/>
-      <c r="B8" s="170"/>
-      <c r="C8" s="122">
+        <v>5</v>
+      </c>
+      <c r="B6" s="174">
+        <f>SUM(Cashflow!M50:M62)</f>
+        <v>178936.03870423092</v>
+      </c>
+      <c r="C6" s="174">
+        <f>ABS(SUM(Cashflow!L50:L62))</f>
+        <v>102318.26807857092</v>
+      </c>
+      <c r="D6" s="174">
         <f t="shared" si="1"/>
-        <v>0.13</v>
-      </c>
-      <c r="D8" s="12">
-        <v>244665.13098403567</v>
-      </c>
-      <c r="E8" s="12">
-        <v>287724.2737791746</v>
-      </c>
-      <c r="F8" s="12">
-        <v>330783.41657431342</v>
-      </c>
-      <c r="G8" s="12">
-        <v>373842.55936945241</v>
-      </c>
-      <c r="H8" s="12">
-        <v>416901.70216459117</v>
-      </c>
-      <c r="I8" s="12">
-        <v>459960.84495973017</v>
-      </c>
-      <c r="J8" s="12">
-        <v>503019.98775486916</v>
-      </c>
-      <c r="K8" s="12">
-        <v>546079.13055000803</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A9" s="10"/>
-      <c r="B9" s="170"/>
-      <c r="C9" s="122">
-        <f t="shared" si="1"/>
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="D9" s="12">
-        <v>303881.46671885811</v>
-      </c>
-      <c r="E9" s="12">
-        <v>350252.85126746923</v>
-      </c>
-      <c r="F9" s="12">
-        <v>396624.2358160803</v>
-      </c>
-      <c r="G9" s="12">
-        <v>442995.62036469148</v>
-      </c>
-      <c r="H9" s="12">
-        <v>489367.00491330249</v>
-      </c>
-      <c r="I9" s="12">
-        <v>535738.38946191373</v>
-      </c>
-      <c r="J9" s="12">
-        <v>582109.77401052485</v>
-      </c>
-      <c r="K9" s="12">
-        <v>628481.15855913586</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B10" s="170"/>
-      <c r="C10" s="122">
-        <f t="shared" si="1"/>
-        <v>0.15000000000000002</v>
-      </c>
-      <c r="D10" s="12">
-        <v>363097.80245368037</v>
-      </c>
-      <c r="E10" s="12">
-        <v>412781.4287557638</v>
-      </c>
-      <c r="F10" s="12">
-        <v>462465.05505784717</v>
-      </c>
-      <c r="G10" s="12">
-        <v>512148.68135993078</v>
-      </c>
-      <c r="H10" s="12">
-        <v>561832.30766201403</v>
-      </c>
-      <c r="I10" s="12">
-        <v>611515.93396409741</v>
-      </c>
-      <c r="J10" s="12">
-        <v>661199.5602661809</v>
-      </c>
-      <c r="K10" s="12">
-        <v>710883.18656826427</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B11" s="170"/>
-      <c r="C11" s="122">
-        <f t="shared" si="1"/>
-        <v>0.16000000000000003</v>
-      </c>
-      <c r="D11" s="12">
-        <v>422314.13818850258</v>
-      </c>
-      <c r="E11" s="12">
-        <v>475310.00624405808</v>
-      </c>
-      <c r="F11" s="12">
-        <v>528305.87429961388</v>
-      </c>
-      <c r="G11" s="12">
-        <v>581301.7423551695</v>
-      </c>
-      <c r="H11" s="12">
-        <v>634297.610410725</v>
-      </c>
-      <c r="I11" s="12">
-        <v>687293.4784662805</v>
-      </c>
-      <c r="J11" s="12">
-        <v>740289.34652183624</v>
-      </c>
-      <c r="K11" s="12">
-        <v>793285.21457739174</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B12" s="170"/>
-      <c r="C12" s="122">
-        <f t="shared" si="1"/>
-        <v>0.17000000000000004</v>
-      </c>
-      <c r="D12" s="12">
-        <v>481530.47392332484</v>
-      </c>
-      <c r="E12" s="12">
-        <v>537838.58373235259</v>
-      </c>
-      <c r="F12" s="12">
-        <v>594146.69354138058</v>
-      </c>
-      <c r="G12" s="12">
-        <v>650454.80335040845</v>
-      </c>
-      <c r="H12" s="12">
-        <v>706762.91315943631</v>
-      </c>
-      <c r="I12" s="12">
-        <v>763071.02296846395</v>
-      </c>
-      <c r="J12" s="12">
-        <v>819379.13277749182</v>
-      </c>
-      <c r="K12" s="12">
-        <v>875687.2425865198</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B13" s="170"/>
-      <c r="C13" s="122">
-        <f t="shared" si="1"/>
-        <v>0.18000000000000005</v>
-      </c>
-      <c r="D13" s="12">
-        <v>540746.80965814728</v>
-      </c>
-      <c r="E13" s="12">
-        <v>600367.16122064716</v>
-      </c>
-      <c r="F13" s="12">
-        <v>659987.51278314728</v>
-      </c>
-      <c r="G13" s="12">
-        <v>719607.86434564739</v>
-      </c>
-      <c r="H13" s="12">
-        <v>779228.21590814739</v>
-      </c>
-      <c r="I13" s="12">
-        <v>838848.56747064739</v>
-      </c>
-      <c r="J13" s="12">
-        <v>898468.91903314739</v>
-      </c>
-      <c r="K13" s="12">
-        <v>958089.27059564739</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B14" s="170"/>
-      <c r="C14" s="122">
-        <f t="shared" si="1"/>
-        <v>0.19000000000000006</v>
-      </c>
-      <c r="D14" s="12">
-        <v>599963.1453929696</v>
-      </c>
-      <c r="E14" s="12">
-        <v>662895.73870894173</v>
-      </c>
-      <c r="F14" s="12">
-        <v>725828.3320249141</v>
-      </c>
-      <c r="G14" s="12">
-        <v>788760.92534088634</v>
-      </c>
-      <c r="H14" s="12">
-        <v>851693.51865685871</v>
-      </c>
-      <c r="I14" s="12">
-        <v>914626.11197283107</v>
-      </c>
-      <c r="J14" s="12">
-        <v>977558.7052888032</v>
-      </c>
-      <c r="K14" s="12">
-        <v>1040491.2986047756</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B15" s="170"/>
-      <c r="C15" s="122">
-        <f t="shared" si="1"/>
-        <v>0.20000000000000007</v>
-      </c>
-      <c r="D15" s="12">
-        <v>659179.48112779169</v>
-      </c>
-      <c r="E15" s="12">
-        <v>725424.31619723607</v>
-      </c>
-      <c r="F15" s="12">
-        <v>791669.15126668103</v>
-      </c>
-      <c r="G15" s="12">
-        <v>857913.98633612553</v>
-      </c>
-      <c r="H15" s="12">
-        <v>924158.82140557002</v>
-      </c>
-      <c r="I15" s="12">
-        <v>990403.65647501452</v>
-      </c>
-      <c r="J15" s="12">
-        <v>1056648.491544459</v>
-      </c>
-      <c r="K15" s="12">
-        <v>1122893.3266139037</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>198</v>
+        <v>168525.42819888069</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B5:B15"/>
-    <mergeCell ref="D3:K3"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>